<commit_message>
Add series/shunt L or C calculation
</commit_message>
<xml_diff>
--- a/Autotransformer_UnUn_AirCore_Calculator.xlsx
+++ b/Autotransformer_UnUn_AirCore_Calculator.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="137">
   <si>
     <t xml:space="preserve">✦  AIR-CORE AUTOTRANSFORMER UnUn CALCULATOR  ✦</t>
   </si>
@@ -357,6 +357,101 @@
   </si>
   <si>
     <t xml:space="preserve">Compare L vs L_min</t>
+  </si>
+  <si>
+    <t xml:space="preserve">✦  COMPENSATION NETWORK CALCULATOR  ✦</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Series &amp; Shunt L/C to cancel residual reactance at each tap — referenced to 50Ω system</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HOW TO READ THIS TABLE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Series L/C: place component in series with the feed line at the tap — cancels reflected reactance seen at that tap port.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shunt L/C:  place component to ground at the tap — cancels the susceptance seen at that tap port.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Positive X (inductive load): series C or shunt C cancels.  Negative X (capacitive load): series L or shunt L cancels.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Values are computed for the tap frequency shown. Component Q and self-resonance should be verified for your operating frequency.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tap 1 (X = 0): no compensation needed — values show "—" automatically.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Freq
+(MHz)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R_tap
+(Ω)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">X_tap
+(Ω)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phase
+(°)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Series L
+(µH)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Series C
+(pF)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shunt L
+(µH)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shunt C
+(pF)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COMPONENT SELECTION GUIDE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Series topology</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Component placed in series with the line at the tap port. Best when source impedance is known and fixed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shunt topology</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Component placed from tap port to ground. Best when line Z is nearly correct but susceptance must be tuned out.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">X = 0 (— shown)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Load is purely resistive — autotransformer alone provides a perfect match. No compensation required.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tolerance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Use ±5% or better components. At HF, stray lead inductance (~5–20 nH) may need to be subtracted from L values.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capacitor type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Use NP0/C0G ceramic or silver-mica capacitors for HF stability. Avoid X7R at RF frequencies.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inductor type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Use air-core solenoid or toroid (T-material) for series inductors. Ensure SRF &gt;&gt; operating frequency.</t>
   </si>
 </sst>
 </file>
@@ -375,7 +470,7 @@
     <numFmt numFmtId="172" formatCode="0.00"/>
     <numFmt numFmtId="173" formatCode="0.0"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -452,8 +547,61 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="12"/>
+      <color rgb="FFFFD700"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i val="true"/>
+      <sz val="10"/>
+      <color rgb="FF8EA9C1"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF404040"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="9"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="9"/>
+      <color rgb="FF1F3864"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -463,19 +611,19 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1A2D40"/>
-        <bgColor rgb="FF003366"/>
+        <bgColor rgb="FF1F3864"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1F5C8B"/>
-        <bgColor rgb="FF008080"/>
+        <bgColor rgb="FF2E4A6B"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
-        <bgColor rgb="FFF0F8FF"/>
+        <bgColor rgb="FFEAF0FB"/>
       </patternFill>
     </fill>
     <fill>
@@ -499,13 +647,31 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD6E8F5"/>
-        <bgColor rgb="FFF2F2F2"/>
+        <bgColor rgb="FFEAF0FB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE8A020"/>
-        <bgColor rgb="FFFFCC00"/>
+        <bgColor rgb="FFFF8080"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F3864"/>
+        <bgColor rgb="FF1A2D40"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2E4A6B"/>
+        <bgColor rgb="FF1F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEAF0FB"/>
+        <bgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -558,7 +724,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="46">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -643,55 +809,23 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="170" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="171" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="172" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="172" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="173" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="173" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -711,14 +845,6 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="172" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -733,6 +859,54 @@
     </xf>
     <xf numFmtId="171" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="11" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="16" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="16" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="16" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="16" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -762,7 +936,7 @@
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FFC0C0C0"/>
       <rgbColor rgb="FF808080"/>
-      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FF8EA9C1"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FFFFF9E6"/>
       <rgbColor rgb="FFD6E8F5"/>
@@ -779,9 +953,9 @@
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
+      <rgbColor rgb="FFEAF0FB"/>
+      <rgbColor rgb="FFF2F2F2"/>
       <rgbColor rgb="FFF0F8FF"/>
-      <rgbColor rgb="FFF2F2F2"/>
-      <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
@@ -789,19 +963,19 @@
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
-      <rgbColor rgb="FFFFCC00"/>
+      <rgbColor rgb="FFFFD700"/>
       <rgbColor rgb="FFE8A020"/>
       <rgbColor rgb="FFFF6600"/>
       <rgbColor rgb="FF555555"/>
       <rgbColor rgb="FFAAAAAA"/>
-      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF1F3864"/>
       <rgbColor rgb="FF339966"/>
       <rgbColor rgb="FF003300"/>
-      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FF1A2D40"/>
       <rgbColor rgb="FF993300"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FF333399"/>
-      <rgbColor rgb="FF1A2D40"/>
+      <rgbColor rgb="FF2E4A6B"/>
+      <rgbColor rgb="FF404040"/>
     </indexedColors>
   </colors>
 </styleSheet>
@@ -1503,98 +1677,98 @@
       <c r="D30" s="4"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="12" t="s">
+      <c r="B31" s="6" t="s">
         <v>32</v>
       </c>
       <c r="C31" s="21" t="n">
         <f aca="false">C7</f>
         <v>50</v>
       </c>
-      <c r="D31" s="22" t="s">
+      <c r="D31" s="8" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B32" s="12" t="s">
+      <c r="B32" s="6" t="s">
         <v>33</v>
       </c>
       <c r="C32" s="21" t="n">
         <f aca="false">IFERROR(aggregate(15,6,C15:C25*(1/(H15:H25="YES")),1),MIN(C15:C25))</f>
         <v>7.2</v>
       </c>
-      <c r="D32" s="22" t="s">
+      <c r="D32" s="8" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B33" s="12" t="s">
+      <c r="B33" s="6" t="s">
         <v>35</v>
       </c>
       <c r="C33" s="21" t="n">
         <f aca="false">C8</f>
         <v>0.45</v>
       </c>
-      <c r="D33" s="22" t="s">
+      <c r="D33" s="8" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B34" s="12" t="s">
+      <c r="B34" s="6" t="s">
         <v>36</v>
       </c>
       <c r="C34" s="21" t="n">
         <f aca="false">C11</f>
         <v>20</v>
       </c>
-      <c r="D34" s="22" t="s">
+      <c r="D34" s="8" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B35" s="12" t="s">
+      <c r="B35" s="6" t="s">
         <v>38</v>
       </c>
       <c r="C35" s="21" t="n">
         <f aca="false">C10</f>
         <v>4</v>
       </c>
-      <c r="D35" s="22" t="s">
+      <c r="D35" s="8" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B36" s="12" t="s">
+      <c r="B36" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="C36" s="23" t="n">
+      <c r="C36" s="22" t="n">
         <f aca="false">I71</f>
         <v>4134.33593212417</v>
       </c>
-      <c r="D36" s="22" t="s">
+      <c r="D36" s="8" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B37" s="12" t="s">
+      <c r="B37" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="C37" s="24" t="n">
+      <c r="C37" s="23" t="n">
         <f aca="false">IFERROR(C115,"—")</f>
         <v>35.9977335339286</v>
       </c>
-      <c r="D37" s="22" t="s">
+      <c r="D37" s="8" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B38" s="12" t="s">
+      <c r="B38" s="6" t="s">
         <v>42</v>
       </c>
       <c r="C38" s="21" t="str">
         <f aca="false">IFERROR(C118,"—")</f>
         <v>✔ YES</v>
       </c>
-      <c r="D38" s="22"/>
+      <c r="D38" s="8"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B40" s="4" t="s">
@@ -1639,408 +1813,408 @@
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B42" s="25" t="n">
+      <c r="B42" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="C42" s="26" t="n">
+      <c r="C42" s="18" t="n">
         <f aca="false">C15</f>
         <v>7.2</v>
       </c>
-      <c r="D42" s="27" t="n">
+      <c r="D42" s="16" t="n">
         <f aca="false">F15</f>
         <v>200</v>
       </c>
-      <c r="E42" s="28" t="n">
+      <c r="E42" s="17" t="n">
         <f aca="false">G15</f>
         <v>0</v>
       </c>
-      <c r="F42" s="29" t="n">
+      <c r="F42" s="19" t="n">
         <f aca="false">D59</f>
         <v>2</v>
       </c>
-      <c r="G42" s="30" t="n">
+      <c r="G42" s="11" t="n">
         <f aca="false">E59</f>
         <v>40</v>
       </c>
-      <c r="H42" s="31" t="n">
+      <c r="H42" s="24" t="n">
         <f aca="false">F78</f>
         <v>1</v>
       </c>
-      <c r="I42" s="32" t="n">
+      <c r="I42" s="25" t="n">
         <f aca="false">G78</f>
         <v>180</v>
       </c>
-      <c r="J42" s="31" t="n">
+      <c r="J42" s="24" t="n">
         <f aca="false">I78</f>
         <v>0</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B43" s="33" t="n">
+      <c r="B43" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="C43" s="26" t="n">
+      <c r="C43" s="18" t="n">
         <f aca="false">C16</f>
         <v>10</v>
       </c>
-      <c r="D43" s="27" t="n">
+      <c r="D43" s="16" t="n">
         <f aca="false">F16</f>
         <v>316.227766016838</v>
       </c>
-      <c r="E43" s="28" t="n">
+      <c r="E43" s="17" t="n">
         <f aca="false">G16</f>
         <v>18.434948822922</v>
       </c>
-      <c r="F43" s="29" t="n">
+      <c r="F43" s="19" t="n">
         <f aca="false">D60</f>
         <v>2.51486685936587</v>
       </c>
-      <c r="G43" s="30" t="n">
+      <c r="G43" s="11" t="n">
         <f aca="false">E60</f>
         <v>50</v>
       </c>
-      <c r="H43" s="31" t="n">
+      <c r="H43" s="24" t="n">
         <f aca="false">F79</f>
         <v>1.38742588672279</v>
       </c>
-      <c r="I43" s="32" t="n">
+      <c r="I43" s="25" t="n">
         <f aca="false">G79</f>
         <v>15.7948252576199</v>
       </c>
-      <c r="J43" s="31" t="n">
+      <c r="J43" s="24" t="n">
         <f aca="false">I79</f>
         <v>2.6334038989724</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B44" s="25" t="n">
+      <c r="B44" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="C44" s="26" t="n">
+      <c r="C44" s="18" t="n">
         <f aca="false">C17</f>
         <v>18</v>
       </c>
-      <c r="D44" s="27" t="n">
+      <c r="D44" s="16" t="n">
         <f aca="false">F17</f>
         <v>457.055795281058</v>
       </c>
-      <c r="E44" s="28" t="n">
+      <c r="E44" s="17" t="n">
         <f aca="false">G17</f>
         <v>-10.0805979875423</v>
       </c>
-      <c r="F44" s="29" t="n">
+      <c r="F44" s="19" t="n">
         <f aca="false">D61</f>
         <v>3.02342784031985</v>
       </c>
-      <c r="G44" s="30" t="n">
+      <c r="G44" s="11" t="n">
         <f aca="false">E61</f>
         <v>60</v>
       </c>
-      <c r="H44" s="31" t="n">
+      <c r="H44" s="24" t="n">
         <f aca="false">F80</f>
         <v>1.19345732284679</v>
       </c>
-      <c r="I44" s="32" t="n">
+      <c r="I44" s="25" t="n">
         <f aca="false">G80</f>
         <v>21.0908803086925</v>
       </c>
-      <c r="J44" s="31" t="n">
+      <c r="J44" s="24" t="n">
         <f aca="false">I80</f>
         <v>0.777878860128034</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B45" s="33" t="n">
+      <c r="B45" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="C45" s="26" t="n">
+      <c r="C45" s="18" t="n">
         <f aca="false">C18</f>
         <v>28</v>
       </c>
-      <c r="D45" s="27" t="n">
+      <c r="D45" s="16" t="n">
         <f aca="false">F18</f>
         <v>800</v>
       </c>
-      <c r="E45" s="28" t="n">
+      <c r="E45" s="17" t="n">
         <f aca="false">G18</f>
         <v>0</v>
       </c>
-      <c r="F45" s="29" t="n">
+      <c r="F45" s="19" t="n">
         <f aca="false">D62</f>
         <v>4</v>
       </c>
-      <c r="G45" s="30" t="n">
+      <c r="G45" s="11" t="n">
         <f aca="false">E62</f>
         <v>80</v>
       </c>
-      <c r="H45" s="31" t="n">
+      <c r="H45" s="24" t="n">
         <f aca="false">F81</f>
         <v>1</v>
       </c>
-      <c r="I45" s="32" t="n">
+      <c r="I45" s="25" t="n">
         <f aca="false">G81</f>
         <v>180</v>
       </c>
-      <c r="J45" s="31" t="n">
+      <c r="J45" s="24" t="n">
         <f aca="false">I81</f>
         <v>0</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B46" s="25" t="n">
+      <c r="B46" s="13" t="n">
         <v>5</v>
       </c>
-      <c r="C46" s="26" t="n">
+      <c r="C46" s="18" t="n">
         <f aca="false">C19</f>
         <v>0</v>
       </c>
-      <c r="D46" s="26" t="str">
+      <c r="D46" s="18" t="str">
         <f aca="false">F19</f>
         <v/>
       </c>
-      <c r="E46" s="26" t="str">
+      <c r="E46" s="18" t="str">
         <f aca="false">G19</f>
         <v/>
       </c>
-      <c r="F46" s="26" t="str">
+      <c r="F46" s="18" t="str">
         <f aca="false">D63</f>
         <v/>
       </c>
-      <c r="G46" s="26" t="str">
+      <c r="G46" s="18" t="str">
         <f aca="false">E63</f>
         <v/>
       </c>
-      <c r="H46" s="26" t="str">
+      <c r="H46" s="18" t="str">
         <f aca="false">F82</f>
         <v/>
       </c>
-      <c r="I46" s="26" t="str">
+      <c r="I46" s="18" t="str">
         <f aca="false">G82</f>
         <v/>
       </c>
-      <c r="J46" s="26" t="str">
+      <c r="J46" s="18" t="str">
         <f aca="false">I82</f>
         <v/>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B47" s="33" t="n">
+      <c r="B47" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="C47" s="26" t="n">
+      <c r="C47" s="18" t="n">
         <f aca="false">C20</f>
         <v>0</v>
       </c>
-      <c r="D47" s="26" t="str">
+      <c r="D47" s="18" t="str">
         <f aca="false">F20</f>
         <v/>
       </c>
-      <c r="E47" s="26" t="str">
+      <c r="E47" s="18" t="str">
         <f aca="false">G20</f>
         <v/>
       </c>
-      <c r="F47" s="26" t="str">
+      <c r="F47" s="18" t="str">
         <f aca="false">D64</f>
         <v/>
       </c>
-      <c r="G47" s="26" t="str">
+      <c r="G47" s="18" t="str">
         <f aca="false">E64</f>
         <v/>
       </c>
-      <c r="H47" s="26" t="str">
+      <c r="H47" s="18" t="str">
         <f aca="false">F83</f>
         <v/>
       </c>
-      <c r="I47" s="26" t="str">
+      <c r="I47" s="18" t="str">
         <f aca="false">G83</f>
         <v/>
       </c>
-      <c r="J47" s="26" t="str">
+      <c r="J47" s="18" t="str">
         <f aca="false">I83</f>
         <v/>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B48" s="25" t="n">
+      <c r="B48" s="13" t="n">
         <v>7</v>
       </c>
-      <c r="C48" s="26" t="n">
+      <c r="C48" s="18" t="n">
         <f aca="false">C21</f>
         <v>0</v>
       </c>
-      <c r="D48" s="26" t="str">
+      <c r="D48" s="18" t="str">
         <f aca="false">F21</f>
         <v/>
       </c>
-      <c r="E48" s="26" t="str">
+      <c r="E48" s="18" t="str">
         <f aca="false">G21</f>
         <v/>
       </c>
-      <c r="F48" s="26" t="str">
+      <c r="F48" s="18" t="str">
         <f aca="false">D65</f>
         <v/>
       </c>
-      <c r="G48" s="26" t="str">
+      <c r="G48" s="18" t="str">
         <f aca="false">E65</f>
         <v/>
       </c>
-      <c r="H48" s="26" t="str">
+      <c r="H48" s="18" t="str">
         <f aca="false">F84</f>
         <v/>
       </c>
-      <c r="I48" s="26" t="str">
+      <c r="I48" s="18" t="str">
         <f aca="false">G84</f>
         <v/>
       </c>
-      <c r="J48" s="26" t="str">
+      <c r="J48" s="18" t="str">
         <f aca="false">I84</f>
         <v/>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B49" s="33" t="n">
+      <c r="B49" s="20" t="n">
         <v>8</v>
       </c>
-      <c r="C49" s="26" t="n">
+      <c r="C49" s="18" t="n">
         <f aca="false">C22</f>
         <v>0</v>
       </c>
-      <c r="D49" s="26" t="str">
+      <c r="D49" s="18" t="str">
         <f aca="false">F22</f>
         <v/>
       </c>
-      <c r="E49" s="26" t="str">
+      <c r="E49" s="18" t="str">
         <f aca="false">G22</f>
         <v/>
       </c>
-      <c r="F49" s="26" t="str">
+      <c r="F49" s="18" t="str">
         <f aca="false">D66</f>
         <v/>
       </c>
-      <c r="G49" s="26" t="str">
+      <c r="G49" s="18" t="str">
         <f aca="false">E66</f>
         <v/>
       </c>
-      <c r="H49" s="26" t="str">
+      <c r="H49" s="18" t="str">
         <f aca="false">F85</f>
         <v/>
       </c>
-      <c r="I49" s="26" t="str">
+      <c r="I49" s="18" t="str">
         <f aca="false">G85</f>
         <v/>
       </c>
-      <c r="J49" s="26" t="str">
+      <c r="J49" s="18" t="str">
         <f aca="false">I85</f>
         <v/>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B50" s="25" t="n">
+      <c r="B50" s="13" t="n">
         <v>9</v>
       </c>
-      <c r="C50" s="26" t="n">
+      <c r="C50" s="18" t="n">
         <f aca="false">C23</f>
         <v>0</v>
       </c>
-      <c r="D50" s="26" t="str">
+      <c r="D50" s="18" t="str">
         <f aca="false">F23</f>
         <v/>
       </c>
-      <c r="E50" s="26" t="str">
+      <c r="E50" s="18" t="str">
         <f aca="false">G23</f>
         <v/>
       </c>
-      <c r="F50" s="26" t="str">
+      <c r="F50" s="18" t="str">
         <f aca="false">D67</f>
         <v/>
       </c>
-      <c r="G50" s="26" t="str">
+      <c r="G50" s="18" t="str">
         <f aca="false">E67</f>
         <v/>
       </c>
-      <c r="H50" s="26" t="str">
+      <c r="H50" s="18" t="str">
         <f aca="false">F86</f>
         <v/>
       </c>
-      <c r="I50" s="26" t="str">
+      <c r="I50" s="18" t="str">
         <f aca="false">G86</f>
         <v/>
       </c>
-      <c r="J50" s="26" t="str">
+      <c r="J50" s="18" t="str">
         <f aca="false">I86</f>
         <v/>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B51" s="33" t="n">
+      <c r="B51" s="20" t="n">
         <v>10</v>
       </c>
-      <c r="C51" s="26" t="n">
+      <c r="C51" s="18" t="n">
         <f aca="false">C24</f>
         <v>0</v>
       </c>
-      <c r="D51" s="26" t="str">
+      <c r="D51" s="18" t="str">
         <f aca="false">F24</f>
         <v/>
       </c>
-      <c r="E51" s="26" t="str">
+      <c r="E51" s="18" t="str">
         <f aca="false">G24</f>
         <v/>
       </c>
-      <c r="F51" s="26" t="str">
+      <c r="F51" s="18" t="str">
         <f aca="false">D68</f>
         <v/>
       </c>
-      <c r="G51" s="26" t="str">
+      <c r="G51" s="18" t="str">
         <f aca="false">E68</f>
         <v/>
       </c>
-      <c r="H51" s="26" t="str">
+      <c r="H51" s="18" t="str">
         <f aca="false">F87</f>
         <v/>
       </c>
-      <c r="I51" s="26" t="str">
+      <c r="I51" s="18" t="str">
         <f aca="false">G87</f>
         <v/>
       </c>
-      <c r="J51" s="26" t="str">
+      <c r="J51" s="18" t="str">
         <f aca="false">I87</f>
         <v/>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B52" s="25" t="n">
+      <c r="B52" s="13" t="n">
         <v>11</v>
       </c>
-      <c r="C52" s="26" t="n">
+      <c r="C52" s="18" t="n">
         <f aca="false">C25</f>
         <v>0</v>
       </c>
-      <c r="D52" s="26" t="str">
+      <c r="D52" s="18" t="str">
         <f aca="false">F25</f>
         <v/>
       </c>
-      <c r="E52" s="26" t="str">
+      <c r="E52" s="18" t="str">
         <f aca="false">G25</f>
         <v/>
       </c>
-      <c r="F52" s="26" t="str">
+      <c r="F52" s="18" t="str">
         <f aca="false">D69</f>
         <v/>
       </c>
-      <c r="G52" s="26" t="str">
+      <c r="G52" s="18" t="str">
         <f aca="false">E69</f>
         <v/>
       </c>
-      <c r="H52" s="26" t="str">
+      <c r="H52" s="18" t="str">
         <f aca="false">F88</f>
         <v/>
       </c>
-      <c r="I52" s="26" t="str">
+      <c r="I52" s="18" t="str">
         <f aca="false">G88</f>
         <v/>
       </c>
-      <c r="J52" s="26" t="str">
+      <c r="J52" s="18" t="str">
         <f aca="false">I88</f>
         <v/>
       </c>
@@ -2133,7 +2307,7 @@
         <f aca="false">IF(E59&lt;&gt;"",E59,"")</f>
         <v>40</v>
       </c>
-      <c r="G59" s="34" t="n">
+      <c r="G59" s="26" t="n">
         <f aca="false">IF(F59&lt;&gt;"",F59*PI()*($C$9+$C$8),"")</f>
         <v>2067.16796606208</v>
       </c>
@@ -2141,7 +2315,7 @@
         <f aca="false">IF(G59&lt;&gt;"",G59*4*0.00000001724*1000000/(PI()*$C$8^2),"")</f>
         <v>224.077432098765</v>
       </c>
-      <c r="I59" s="34" t="n">
+      <c r="I59" s="26" t="n">
         <f aca="false">IF(G59&lt;&gt;"",G59,"")</f>
         <v>2067.16796606208</v>
       </c>
@@ -2170,7 +2344,7 @@
         <f aca="false">IF(AND(E60&lt;&gt;"",E59&lt;&gt;""),E60-E59,IF(E60&lt;&gt;"",E60,""))</f>
         <v>10</v>
       </c>
-      <c r="G60" s="34" t="n">
+      <c r="G60" s="26" t="n">
         <f aca="false">IF(F60&lt;&gt;"",F60*PI()*($C$9+$C$8),"")</f>
         <v>516.791991515521</v>
       </c>
@@ -2178,7 +2352,7 @@
         <f aca="false">IF(G60&lt;&gt;"",G60*4*0.00000001724*1000000/(PI()*$C$8^2),"")</f>
         <v>56.0193580246914</v>
       </c>
-      <c r="I60" s="34" t="n">
+      <c r="I60" s="26" t="n">
         <f aca="false">IF(G60&lt;&gt;"",SUM(G59:G60),"")</f>
         <v>2583.9599575776</v>
       </c>
@@ -2207,7 +2381,7 @@
         <f aca="false">IF(AND(E61&lt;&gt;"",E60&lt;&gt;""),E61-E60,IF(E61&lt;&gt;"",E61,""))</f>
         <v>10</v>
       </c>
-      <c r="G61" s="34" t="n">
+      <c r="G61" s="26" t="n">
         <f aca="false">IF(F61&lt;&gt;"",F61*PI()*($C$9+$C$8),"")</f>
         <v>516.791991515521</v>
       </c>
@@ -2215,7 +2389,7 @@
         <f aca="false">IF(G61&lt;&gt;"",G61*4*0.00000001724*1000000/(PI()*$C$8^2),"")</f>
         <v>56.0193580246914</v>
       </c>
-      <c r="I61" s="34" t="n">
+      <c r="I61" s="26" t="n">
         <f aca="false">IF(G61&lt;&gt;"",SUM(G59:G61),"")</f>
         <v>3100.75194909313</v>
       </c>
@@ -2244,7 +2418,7 @@
         <f aca="false">IF(AND(E62&lt;&gt;"",E61&lt;&gt;""),E62-E61,IF(E62&lt;&gt;"",E62,""))</f>
         <v>20</v>
       </c>
-      <c r="G62" s="34" t="n">
+      <c r="G62" s="26" t="n">
         <f aca="false">IF(F62&lt;&gt;"",F62*PI()*($C$9+$C$8),"")</f>
         <v>1033.58398303104</v>
       </c>
@@ -2252,7 +2426,7 @@
         <f aca="false">IF(G62&lt;&gt;"",G62*4*0.00000001724*1000000/(PI()*$C$8^2),"")</f>
         <v>112.038716049383</v>
       </c>
-      <c r="I62" s="34" t="n">
+      <c r="I62" s="26" t="n">
         <f aca="false">IF(G62&lt;&gt;"",SUM(G59:G62),"")</f>
         <v>4134.33593212417</v>
       </c>
@@ -2281,7 +2455,7 @@
         <f aca="false">IF(AND(E63&lt;&gt;"",E62&lt;&gt;""),E63-E62,IF(E63&lt;&gt;"",E63,""))</f>
         <v/>
       </c>
-      <c r="G63" s="34" t="str">
+      <c r="G63" s="26" t="str">
         <f aca="false">IF(F63&lt;&gt;"",F63*PI()*($C$9+$C$8),"")</f>
         <v/>
       </c>
@@ -2289,7 +2463,7 @@
         <f aca="false">IF(G63&lt;&gt;"",G63*4*0.00000001724*1000000/(PI()*$C$8^2),"")</f>
         <v/>
       </c>
-      <c r="I63" s="34" t="str">
+      <c r="I63" s="26" t="str">
         <f aca="false">IF(G63&lt;&gt;"",SUM(G59:G63),"")</f>
         <v/>
       </c>
@@ -2318,7 +2492,7 @@
         <f aca="false">IF(AND(E64&lt;&gt;"",E63&lt;&gt;""),E64-E63,IF(E64&lt;&gt;"",E64,""))</f>
         <v/>
       </c>
-      <c r="G64" s="34" t="str">
+      <c r="G64" s="26" t="str">
         <f aca="false">IF(F64&lt;&gt;"",F64*PI()*($C$9+$C$8),"")</f>
         <v/>
       </c>
@@ -2326,7 +2500,7 @@
         <f aca="false">IF(G64&lt;&gt;"",G64*4*0.00000001724*1000000/(PI()*$C$8^2),"")</f>
         <v/>
       </c>
-      <c r="I64" s="34" t="str">
+      <c r="I64" s="26" t="str">
         <f aca="false">IF(G64&lt;&gt;"",SUM(G59:G64),"")</f>
         <v/>
       </c>
@@ -2355,7 +2529,7 @@
         <f aca="false">IF(AND(E65&lt;&gt;"",E64&lt;&gt;""),E65-E64,IF(E65&lt;&gt;"",E65,""))</f>
         <v/>
       </c>
-      <c r="G65" s="34" t="str">
+      <c r="G65" s="26" t="str">
         <f aca="false">IF(F65&lt;&gt;"",F65*PI()*($C$9+$C$8),"")</f>
         <v/>
       </c>
@@ -2363,7 +2537,7 @@
         <f aca="false">IF(G65&lt;&gt;"",G65*4*0.00000001724*1000000/(PI()*$C$8^2),"")</f>
         <v/>
       </c>
-      <c r="I65" s="34" t="str">
+      <c r="I65" s="26" t="str">
         <f aca="false">IF(G65&lt;&gt;"",SUM(G59:G65),"")</f>
         <v/>
       </c>
@@ -2392,7 +2566,7 @@
         <f aca="false">IF(AND(E66&lt;&gt;"",E65&lt;&gt;""),E66-E65,IF(E66&lt;&gt;"",E66,""))</f>
         <v/>
       </c>
-      <c r="G66" s="34" t="str">
+      <c r="G66" s="26" t="str">
         <f aca="false">IF(F66&lt;&gt;"",F66*PI()*($C$9+$C$8),"")</f>
         <v/>
       </c>
@@ -2400,7 +2574,7 @@
         <f aca="false">IF(G66&lt;&gt;"",G66*4*0.00000001724*1000000/(PI()*$C$8^2),"")</f>
         <v/>
       </c>
-      <c r="I66" s="34" t="str">
+      <c r="I66" s="26" t="str">
         <f aca="false">IF(G66&lt;&gt;"",SUM(G59:G66),"")</f>
         <v/>
       </c>
@@ -2429,7 +2603,7 @@
         <f aca="false">IF(AND(E67&lt;&gt;"",E66&lt;&gt;""),E67-E66,IF(E67&lt;&gt;"",E67,""))</f>
         <v/>
       </c>
-      <c r="G67" s="34" t="str">
+      <c r="G67" s="26" t="str">
         <f aca="false">IF(F67&lt;&gt;"",F67*PI()*($C$9+$C$8),"")</f>
         <v/>
       </c>
@@ -2437,7 +2611,7 @@
         <f aca="false">IF(G67&lt;&gt;"",G67*4*0.00000001724*1000000/(PI()*$C$8^2),"")</f>
         <v/>
       </c>
-      <c r="I67" s="34" t="str">
+      <c r="I67" s="26" t="str">
         <f aca="false">IF(G67&lt;&gt;"",SUM(G59:G67),"")</f>
         <v/>
       </c>
@@ -2466,7 +2640,7 @@
         <f aca="false">IF(AND(E68&lt;&gt;"",E67&lt;&gt;""),E68-E67,IF(E68&lt;&gt;"",E68,""))</f>
         <v/>
       </c>
-      <c r="G68" s="34" t="str">
+      <c r="G68" s="26" t="str">
         <f aca="false">IF(F68&lt;&gt;"",F68*PI()*($C$9+$C$8),"")</f>
         <v/>
       </c>
@@ -2474,7 +2648,7 @@
         <f aca="false">IF(G68&lt;&gt;"",G68*4*0.00000001724*1000000/(PI()*$C$8^2),"")</f>
         <v/>
       </c>
-      <c r="I68" s="34" t="str">
+      <c r="I68" s="26" t="str">
         <f aca="false">IF(G68&lt;&gt;"",SUM(G59:G68),"")</f>
         <v/>
       </c>
@@ -2503,7 +2677,7 @@
         <f aca="false">IF(AND(E69&lt;&gt;"",E68&lt;&gt;""),E69-E68,IF(E69&lt;&gt;"",E69,""))</f>
         <v/>
       </c>
-      <c r="G69" s="34" t="str">
+      <c r="G69" s="26" t="str">
         <f aca="false">IF(F69&lt;&gt;"",F69*PI()*($C$9+$C$8),"")</f>
         <v/>
       </c>
@@ -2511,7 +2685,7 @@
         <f aca="false">IF(G69&lt;&gt;"",G69*4*0.00000001724*1000000/(PI()*$C$8^2),"")</f>
         <v/>
       </c>
-      <c r="I69" s="34" t="str">
+      <c r="I69" s="26" t="str">
         <f aca="false">IF(G69&lt;&gt;"",SUM(G59:G69),"")</f>
         <v/>
       </c>
@@ -2521,20 +2695,20 @@
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B71" s="35" t="s">
+      <c r="B71" s="27" t="s">
         <v>60</v>
       </c>
-      <c r="C71" s="35"/>
-      <c r="D71" s="35"/>
+      <c r="C71" s="27"/>
+      <c r="D71" s="27"/>
       <c r="E71" s="11" t="n">
         <f aca="false">IFERROR(MAX(E59:E69),"")</f>
         <v>80</v>
       </c>
-      <c r="H71" s="36" t="n">
+      <c r="H71" s="28" t="n">
         <f aca="false">IFERROR(SUM(H59:H69),"")</f>
         <v>448.154864197531</v>
       </c>
-      <c r="I71" s="37" t="n">
+      <c r="I71" s="29" t="n">
         <f aca="false">IFERROR(MAX(I59:I69),"")</f>
         <v>4134.33593212417</v>
       </c>
@@ -2613,23 +2787,23 @@
         <f aca="false">F15</f>
         <v>200</v>
       </c>
-      <c r="E78" s="38" t="n">
+      <c r="E78" s="25" t="n">
         <f aca="false">G15</f>
         <v>0</v>
       </c>
-      <c r="F78" s="39" t="n">
+      <c r="F78" s="24" t="n">
         <f aca="false">IF(F15&lt;&gt;"",IFERROR((1+SQRT(((IF(ISNUMBER(D15),D15/MAX((F15/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E15),E15/MAX((F15/C7),0.000000001),0))^2)/((IF(ISNUMBER(D15),D15/MAX((F15/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E15),E15/MAX((F15/C7),0.000000001),0))^2)))/(1-SQRT(((IF(ISNUMBER(D15),D15/MAX((F15/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E15),E15/MAX((F15/C7),0.000000001),0))^2)/((IF(ISNUMBER(D15),D15/MAX((F15/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E15),E15/MAX((F15/C7),0.000000001),0))^2))),999),"")</f>
         <v>1</v>
       </c>
-      <c r="G78" s="38" t="n">
+      <c r="G78" s="25" t="n">
         <f aca="false">IF(F15&lt;&gt;"",IFERROR(-20*LOG10(MAX(SQRT(((IF(ISNUMBER(D15),D15/MAX((F15/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E15),E15/MAX((F15/C7),0.000000001),0))^2)/((IF(ISNUMBER(D15),D15/MAX((F15/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E15),E15/MAX((F15/C7),0.000000001),0))^2)),0.000000001)),0),"")</f>
         <v>180</v>
       </c>
-      <c r="H78" s="39" t="n">
+      <c r="H78" s="24" t="n">
         <f aca="false">IF(F15&lt;&gt;"",IFERROR(MAX(0,-10*LOG10(1-((IF(ISNUMBER(D15),D15/MAX((F15/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E15),E15/MAX((F15/C7),0.000000001),0))^2)/((IF(ISNUMBER(D15),D15/MAX((F15/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E15),E15/MAX((F15/C7),0.000000001),0))^2))),0),"")</f>
         <v>-0</v>
       </c>
-      <c r="I78" s="39" t="n">
+      <c r="I78" s="24" t="n">
         <f aca="false">IF(F15&lt;&gt;"",IFERROR(((IF(ISNUMBER(D15),D15/MAX((F15/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E15),E15/MAX((F15/C7),0.000000001),0))^2)/((IF(ISNUMBER(D15),D15/MAX((F15/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E15),E15/MAX((F15/C7),0.000000001),0))^2)*100,0),"")</f>
         <v>0</v>
       </c>
@@ -2646,23 +2820,23 @@
         <f aca="false">F16</f>
         <v>316.227766016838</v>
       </c>
-      <c r="E79" s="38" t="n">
+      <c r="E79" s="25" t="n">
         <f aca="false">G16</f>
         <v>18.434948822922</v>
       </c>
-      <c r="F79" s="39" t="n">
+      <c r="F79" s="24" t="n">
         <f aca="false">IF(F16&lt;&gt;"",IFERROR((1+SQRT(((IF(ISNUMBER(D16),D16/MAX((F16/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E16),E16/MAX((F16/C7),0.000000001),0))^2)/((IF(ISNUMBER(D16),D16/MAX((F16/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E16),E16/MAX((F16/C7),0.000000001),0))^2)))/(1-SQRT(((IF(ISNUMBER(D16),D16/MAX((F16/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E16),E16/MAX((F16/C7),0.000000001),0))^2)/((IF(ISNUMBER(D16),D16/MAX((F16/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E16),E16/MAX((F16/C7),0.000000001),0))^2))),999),"")</f>
         <v>1.38742588672279</v>
       </c>
-      <c r="G79" s="38" t="n">
+      <c r="G79" s="25" t="n">
         <f aca="false">IF(F16&lt;&gt;"",IFERROR(-20*LOG10(MAX(SQRT(((IF(ISNUMBER(D16),D16/MAX((F16/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E16),E16/MAX((F16/C7),0.000000001),0))^2)/((IF(ISNUMBER(D16),D16/MAX((F16/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E16),E16/MAX((F16/C7),0.000000001),0))^2)),0.000000001)),0),"")</f>
         <v>15.7948252576199</v>
       </c>
-      <c r="H79" s="39" t="n">
+      <c r="H79" s="24" t="n">
         <f aca="false">IF(F16&lt;&gt;"",IFERROR(MAX(0,-10*LOG10(1-((IF(ISNUMBER(D16),D16/MAX((F16/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E16),E16/MAX((F16/C7),0.000000001),0))^2)/((IF(ISNUMBER(D16),D16/MAX((F16/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E16),E16/MAX((F16/C7),0.000000001),0))^2))),0),"")</f>
         <v>0.115900124973496</v>
       </c>
-      <c r="I79" s="39" t="n">
+      <c r="I79" s="24" t="n">
         <f aca="false">IF(F16&lt;&gt;"",IFERROR(((IF(ISNUMBER(D16),D16/MAX((F16/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E16),E16/MAX((F16/C7),0.000000001),0))^2)/((IF(ISNUMBER(D16),D16/MAX((F16/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E16),E16/MAX((F16/C7),0.000000001),0))^2)*100,0),"")</f>
         <v>2.6334038989724</v>
       </c>
@@ -2679,23 +2853,23 @@
         <f aca="false">F17</f>
         <v>457.055795281058</v>
       </c>
-      <c r="E80" s="38" t="n">
+      <c r="E80" s="25" t="n">
         <f aca="false">G17</f>
         <v>-10.0805979875423</v>
       </c>
-      <c r="F80" s="39" t="n">
+      <c r="F80" s="24" t="n">
         <f aca="false">IF(F17&lt;&gt;"",IFERROR((1+SQRT(((IF(ISNUMBER(D17),D17/MAX((F17/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E17),E17/MAX((F17/C7),0.000000001),0))^2)/((IF(ISNUMBER(D17),D17/MAX((F17/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E17),E17/MAX((F17/C7),0.000000001),0))^2)))/(1-SQRT(((IF(ISNUMBER(D17),D17/MAX((F17/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E17),E17/MAX((F17/C7),0.000000001),0))^2)/((IF(ISNUMBER(D17),D17/MAX((F17/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E17),E17/MAX((F17/C7),0.000000001),0))^2))),999),"")</f>
         <v>1.19345732284679</v>
       </c>
-      <c r="G80" s="38" t="n">
+      <c r="G80" s="25" t="n">
         <f aca="false">IF(F17&lt;&gt;"",IFERROR(-20*LOG10(MAX(SQRT(((IF(ISNUMBER(D17),D17/MAX((F17/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E17),E17/MAX((F17/C7),0.000000001),0))^2)/((IF(ISNUMBER(D17),D17/MAX((F17/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E17),E17/MAX((F17/C7),0.000000001),0))^2)),0.000000001)),0),"")</f>
         <v>21.0908803086925</v>
       </c>
-      <c r="H80" s="39" t="n">
+      <c r="H80" s="24" t="n">
         <f aca="false">IF(F17&lt;&gt;"",IFERROR(MAX(0,-10*LOG10(1-((IF(ISNUMBER(D17),D17/MAX((F17/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E17),E17/MAX((F17/C7),0.000000001),0))^2)/((IF(ISNUMBER(D17),D17/MAX((F17/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E17),E17/MAX((F17/C7),0.000000001),0))^2))),0),"")</f>
         <v>0.0339149298724391</v>
       </c>
-      <c r="I80" s="39" t="n">
+      <c r="I80" s="24" t="n">
         <f aca="false">IF(F17&lt;&gt;"",IFERROR(((IF(ISNUMBER(D17),D17/MAX((F17/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E17),E17/MAX((F17/C7),0.000000001),0))^2)/((IF(ISNUMBER(D17),D17/MAX((F17/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E17),E17/MAX((F17/C7),0.000000001),0))^2)*100,0),"")</f>
         <v>0.777878860128034</v>
       </c>
@@ -2712,23 +2886,23 @@
         <f aca="false">F18</f>
         <v>800</v>
       </c>
-      <c r="E81" s="38" t="n">
+      <c r="E81" s="25" t="n">
         <f aca="false">G18</f>
         <v>0</v>
       </c>
-      <c r="F81" s="39" t="n">
+      <c r="F81" s="24" t="n">
         <f aca="false">IF(F18&lt;&gt;"",IFERROR((1+SQRT(((IF(ISNUMBER(D18),D18/MAX((F18/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E18),E18/MAX((F18/C7),0.000000001),0))^2)/((IF(ISNUMBER(D18),D18/MAX((F18/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E18),E18/MAX((F18/C7),0.000000001),0))^2)))/(1-SQRT(((IF(ISNUMBER(D18),D18/MAX((F18/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E18),E18/MAX((F18/C7),0.000000001),0))^2)/((IF(ISNUMBER(D18),D18/MAX((F18/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E18),E18/MAX((F18/C7),0.000000001),0))^2))),999),"")</f>
         <v>1</v>
       </c>
-      <c r="G81" s="38" t="n">
+      <c r="G81" s="25" t="n">
         <f aca="false">IF(F18&lt;&gt;"",IFERROR(-20*LOG10(MAX(SQRT(((IF(ISNUMBER(D18),D18/MAX((F18/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E18),E18/MAX((F18/C7),0.000000001),0))^2)/((IF(ISNUMBER(D18),D18/MAX((F18/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E18),E18/MAX((F18/C7),0.000000001),0))^2)),0.000000001)),0),"")</f>
         <v>180</v>
       </c>
-      <c r="H81" s="39" t="n">
+      <c r="H81" s="24" t="n">
         <f aca="false">IF(F18&lt;&gt;"",IFERROR(MAX(0,-10*LOG10(1-((IF(ISNUMBER(D18),D18/MAX((F18/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E18),E18/MAX((F18/C7),0.000000001),0))^2)/((IF(ISNUMBER(D18),D18/MAX((F18/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E18),E18/MAX((F18/C7),0.000000001),0))^2))),0),"")</f>
         <v>-0</v>
       </c>
-      <c r="I81" s="39" t="n">
+      <c r="I81" s="24" t="n">
         <f aca="false">IF(F18&lt;&gt;"",IFERROR(((IF(ISNUMBER(D18),D18/MAX((F18/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E18),E18/MAX((F18/C7),0.000000001),0))^2)/((IF(ISNUMBER(D18),D18/MAX((F18/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E18),E18/MAX((F18/C7),0.000000001),0))^2)*100,0),"")</f>
         <v>0</v>
       </c>
@@ -2745,23 +2919,23 @@
         <f aca="false">F19</f>
         <v/>
       </c>
-      <c r="E82" s="38" t="str">
+      <c r="E82" s="25" t="str">
         <f aca="false">G19</f>
         <v/>
       </c>
-      <c r="F82" s="39" t="str">
+      <c r="F82" s="24" t="str">
         <f aca="false">IF(F19&lt;&gt;"",IFERROR((1+SQRT(((IF(ISNUMBER(D19),D19/MAX((F19/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E19),E19/MAX((F19/C7),0.000000001),0))^2)/((IF(ISNUMBER(D19),D19/MAX((F19/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E19),E19/MAX((F19/C7),0.000000001),0))^2)))/(1-SQRT(((IF(ISNUMBER(D19),D19/MAX((F19/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E19),E19/MAX((F19/C7),0.000000001),0))^2)/((IF(ISNUMBER(D19),D19/MAX((F19/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E19),E19/MAX((F19/C7),0.000000001),0))^2))),999),"")</f>
         <v/>
       </c>
-      <c r="G82" s="38" t="str">
+      <c r="G82" s="25" t="str">
         <f aca="false">IF(F19&lt;&gt;"",IFERROR(-20*LOG10(MAX(SQRT(((IF(ISNUMBER(D19),D19/MAX((F19/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E19),E19/MAX((F19/C7),0.000000001),0))^2)/((IF(ISNUMBER(D19),D19/MAX((F19/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E19),E19/MAX((F19/C7),0.000000001),0))^2)),0.000000001)),0),"")</f>
         <v/>
       </c>
-      <c r="H82" s="39" t="str">
+      <c r="H82" s="24" t="str">
         <f aca="false">IF(F19&lt;&gt;"",IFERROR(MAX(0,-10*LOG10(1-((IF(ISNUMBER(D19),D19/MAX((F19/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E19),E19/MAX((F19/C7),0.000000001),0))^2)/((IF(ISNUMBER(D19),D19/MAX((F19/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E19),E19/MAX((F19/C7),0.000000001),0))^2))),0),"")</f>
         <v/>
       </c>
-      <c r="I82" s="39" t="str">
+      <c r="I82" s="24" t="str">
         <f aca="false">IF(F19&lt;&gt;"",IFERROR(((IF(ISNUMBER(D19),D19/MAX((F19/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E19),E19/MAX((F19/C7),0.000000001),0))^2)/((IF(ISNUMBER(D19),D19/MAX((F19/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E19),E19/MAX((F19/C7),0.000000001),0))^2)*100,0),"")</f>
         <v/>
       </c>
@@ -2778,23 +2952,23 @@
         <f aca="false">F20</f>
         <v/>
       </c>
-      <c r="E83" s="38" t="str">
+      <c r="E83" s="25" t="str">
         <f aca="false">G20</f>
         <v/>
       </c>
-      <c r="F83" s="39" t="str">
+      <c r="F83" s="24" t="str">
         <f aca="false">IF(F20&lt;&gt;"",IFERROR((1+SQRT(((IF(ISNUMBER(D20),D20/MAX((F20/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E20),E20/MAX((F20/C7),0.000000001),0))^2)/((IF(ISNUMBER(D20),D20/MAX((F20/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E20),E20/MAX((F20/C7),0.000000001),0))^2)))/(1-SQRT(((IF(ISNUMBER(D20),D20/MAX((F20/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E20),E20/MAX((F20/C7),0.000000001),0))^2)/((IF(ISNUMBER(D20),D20/MAX((F20/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E20),E20/MAX((F20/C7),0.000000001),0))^2))),999),"")</f>
         <v/>
       </c>
-      <c r="G83" s="38" t="str">
+      <c r="G83" s="25" t="str">
         <f aca="false">IF(F20&lt;&gt;"",IFERROR(-20*LOG10(MAX(SQRT(((IF(ISNUMBER(D20),D20/MAX((F20/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E20),E20/MAX((F20/C7),0.000000001),0))^2)/((IF(ISNUMBER(D20),D20/MAX((F20/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E20),E20/MAX((F20/C7),0.000000001),0))^2)),0.000000001)),0),"")</f>
         <v/>
       </c>
-      <c r="H83" s="39" t="str">
+      <c r="H83" s="24" t="str">
         <f aca="false">IF(F20&lt;&gt;"",IFERROR(MAX(0,-10*LOG10(1-((IF(ISNUMBER(D20),D20/MAX((F20/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E20),E20/MAX((F20/C7),0.000000001),0))^2)/((IF(ISNUMBER(D20),D20/MAX((F20/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E20),E20/MAX((F20/C7),0.000000001),0))^2))),0),"")</f>
         <v/>
       </c>
-      <c r="I83" s="39" t="str">
+      <c r="I83" s="24" t="str">
         <f aca="false">IF(F20&lt;&gt;"",IFERROR(((IF(ISNUMBER(D20),D20/MAX((F20/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E20),E20/MAX((F20/C7),0.000000001),0))^2)/((IF(ISNUMBER(D20),D20/MAX((F20/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E20),E20/MAX((F20/C7),0.000000001),0))^2)*100,0),"")</f>
         <v/>
       </c>
@@ -2811,23 +2985,23 @@
         <f aca="false">F21</f>
         <v/>
       </c>
-      <c r="E84" s="38" t="str">
+      <c r="E84" s="25" t="str">
         <f aca="false">G21</f>
         <v/>
       </c>
-      <c r="F84" s="39" t="str">
+      <c r="F84" s="24" t="str">
         <f aca="false">IF(F21&lt;&gt;"",IFERROR((1+SQRT(((IF(ISNUMBER(D21),D21/MAX((F21/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E21),E21/MAX((F21/C7),0.000000001),0))^2)/((IF(ISNUMBER(D21),D21/MAX((F21/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E21),E21/MAX((F21/C7),0.000000001),0))^2)))/(1-SQRT(((IF(ISNUMBER(D21),D21/MAX((F21/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E21),E21/MAX((F21/C7),0.000000001),0))^2)/((IF(ISNUMBER(D21),D21/MAX((F21/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E21),E21/MAX((F21/C7),0.000000001),0))^2))),999),"")</f>
         <v/>
       </c>
-      <c r="G84" s="38" t="str">
+      <c r="G84" s="25" t="str">
         <f aca="false">IF(F21&lt;&gt;"",IFERROR(-20*LOG10(MAX(SQRT(((IF(ISNUMBER(D21),D21/MAX((F21/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E21),E21/MAX((F21/C7),0.000000001),0))^2)/((IF(ISNUMBER(D21),D21/MAX((F21/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E21),E21/MAX((F21/C7),0.000000001),0))^2)),0.000000001)),0),"")</f>
         <v/>
       </c>
-      <c r="H84" s="39" t="str">
+      <c r="H84" s="24" t="str">
         <f aca="false">IF(F21&lt;&gt;"",IFERROR(MAX(0,-10*LOG10(1-((IF(ISNUMBER(D21),D21/MAX((F21/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E21),E21/MAX((F21/C7),0.000000001),0))^2)/((IF(ISNUMBER(D21),D21/MAX((F21/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E21),E21/MAX((F21/C7),0.000000001),0))^2))),0),"")</f>
         <v/>
       </c>
-      <c r="I84" s="39" t="str">
+      <c r="I84" s="24" t="str">
         <f aca="false">IF(F21&lt;&gt;"",IFERROR(((IF(ISNUMBER(D21),D21/MAX((F21/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E21),E21/MAX((F21/C7),0.000000001),0))^2)/((IF(ISNUMBER(D21),D21/MAX((F21/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E21),E21/MAX((F21/C7),0.000000001),0))^2)*100,0),"")</f>
         <v/>
       </c>
@@ -2844,23 +3018,23 @@
         <f aca="false">F22</f>
         <v/>
       </c>
-      <c r="E85" s="38" t="str">
+      <c r="E85" s="25" t="str">
         <f aca="false">G22</f>
         <v/>
       </c>
-      <c r="F85" s="39" t="str">
+      <c r="F85" s="24" t="str">
         <f aca="false">IF(F22&lt;&gt;"",IFERROR((1+SQRT(((IF(ISNUMBER(D22),D22/MAX((F22/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E22),E22/MAX((F22/C7),0.000000001),0))^2)/((IF(ISNUMBER(D22),D22/MAX((F22/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E22),E22/MAX((F22/C7),0.000000001),0))^2)))/(1-SQRT(((IF(ISNUMBER(D22),D22/MAX((F22/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E22),E22/MAX((F22/C7),0.000000001),0))^2)/((IF(ISNUMBER(D22),D22/MAX((F22/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E22),E22/MAX((F22/C7),0.000000001),0))^2))),999),"")</f>
         <v/>
       </c>
-      <c r="G85" s="38" t="str">
+      <c r="G85" s="25" t="str">
         <f aca="false">IF(F22&lt;&gt;"",IFERROR(-20*LOG10(MAX(SQRT(((IF(ISNUMBER(D22),D22/MAX((F22/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E22),E22/MAX((F22/C7),0.000000001),0))^2)/((IF(ISNUMBER(D22),D22/MAX((F22/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E22),E22/MAX((F22/C7),0.000000001),0))^2)),0.000000001)),0),"")</f>
         <v/>
       </c>
-      <c r="H85" s="39" t="str">
+      <c r="H85" s="24" t="str">
         <f aca="false">IF(F22&lt;&gt;"",IFERROR(MAX(0,-10*LOG10(1-((IF(ISNUMBER(D22),D22/MAX((F22/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E22),E22/MAX((F22/C7),0.000000001),0))^2)/((IF(ISNUMBER(D22),D22/MAX((F22/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E22),E22/MAX((F22/C7),0.000000001),0))^2))),0),"")</f>
         <v/>
       </c>
-      <c r="I85" s="39" t="str">
+      <c r="I85" s="24" t="str">
         <f aca="false">IF(F22&lt;&gt;"",IFERROR(((IF(ISNUMBER(D22),D22/MAX((F22/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E22),E22/MAX((F22/C7),0.000000001),0))^2)/((IF(ISNUMBER(D22),D22/MAX((F22/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E22),E22/MAX((F22/C7),0.000000001),0))^2)*100,0),"")</f>
         <v/>
       </c>
@@ -2877,23 +3051,23 @@
         <f aca="false">F23</f>
         <v/>
       </c>
-      <c r="E86" s="38" t="str">
+      <c r="E86" s="25" t="str">
         <f aca="false">G23</f>
         <v/>
       </c>
-      <c r="F86" s="39" t="str">
+      <c r="F86" s="24" t="str">
         <f aca="false">IF(F23&lt;&gt;"",IFERROR((1+SQRT(((IF(ISNUMBER(D23),D23/MAX((F23/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E23),E23/MAX((F23/C7),0.000000001),0))^2)/((IF(ISNUMBER(D23),D23/MAX((F23/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E23),E23/MAX((F23/C7),0.000000001),0))^2)))/(1-SQRT(((IF(ISNUMBER(D23),D23/MAX((F23/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E23),E23/MAX((F23/C7),0.000000001),0))^2)/((IF(ISNUMBER(D23),D23/MAX((F23/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E23),E23/MAX((F23/C7),0.000000001),0))^2))),999),"")</f>
         <v/>
       </c>
-      <c r="G86" s="38" t="str">
+      <c r="G86" s="25" t="str">
         <f aca="false">IF(F23&lt;&gt;"",IFERROR(-20*LOG10(MAX(SQRT(((IF(ISNUMBER(D23),D23/MAX((F23/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E23),E23/MAX((F23/C7),0.000000001),0))^2)/((IF(ISNUMBER(D23),D23/MAX((F23/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E23),E23/MAX((F23/C7),0.000000001),0))^2)),0.000000001)),0),"")</f>
         <v/>
       </c>
-      <c r="H86" s="39" t="str">
+      <c r="H86" s="24" t="str">
         <f aca="false">IF(F23&lt;&gt;"",IFERROR(MAX(0,-10*LOG10(1-((IF(ISNUMBER(D23),D23/MAX((F23/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E23),E23/MAX((F23/C7),0.000000001),0))^2)/((IF(ISNUMBER(D23),D23/MAX((F23/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E23),E23/MAX((F23/C7),0.000000001),0))^2))),0),"")</f>
         <v/>
       </c>
-      <c r="I86" s="39" t="str">
+      <c r="I86" s="24" t="str">
         <f aca="false">IF(F23&lt;&gt;"",IFERROR(((IF(ISNUMBER(D23),D23/MAX((F23/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E23),E23/MAX((F23/C7),0.000000001),0))^2)/((IF(ISNUMBER(D23),D23/MAX((F23/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E23),E23/MAX((F23/C7),0.000000001),0))^2)*100,0),"")</f>
         <v/>
       </c>
@@ -2910,23 +3084,23 @@
         <f aca="false">F24</f>
         <v/>
       </c>
-      <c r="E87" s="38" t="str">
+      <c r="E87" s="25" t="str">
         <f aca="false">G24</f>
         <v/>
       </c>
-      <c r="F87" s="39" t="str">
+      <c r="F87" s="24" t="str">
         <f aca="false">IF(F24&lt;&gt;"",IFERROR((1+SQRT(((IF(ISNUMBER(D24),D24/MAX((F24/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E24),E24/MAX((F24/C7),0.000000001),0))^2)/((IF(ISNUMBER(D24),D24/MAX((F24/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E24),E24/MAX((F24/C7),0.000000001),0))^2)))/(1-SQRT(((IF(ISNUMBER(D24),D24/MAX((F24/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E24),E24/MAX((F24/C7),0.000000001),0))^2)/((IF(ISNUMBER(D24),D24/MAX((F24/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E24),E24/MAX((F24/C7),0.000000001),0))^2))),999),"")</f>
         <v/>
       </c>
-      <c r="G87" s="38" t="str">
+      <c r="G87" s="25" t="str">
         <f aca="false">IF(F24&lt;&gt;"",IFERROR(-20*LOG10(MAX(SQRT(((IF(ISNUMBER(D24),D24/MAX((F24/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E24),E24/MAX((F24/C7),0.000000001),0))^2)/((IF(ISNUMBER(D24),D24/MAX((F24/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E24),E24/MAX((F24/C7),0.000000001),0))^2)),0.000000001)),0),"")</f>
         <v/>
       </c>
-      <c r="H87" s="39" t="str">
+      <c r="H87" s="24" t="str">
         <f aca="false">IF(F24&lt;&gt;"",IFERROR(MAX(0,-10*LOG10(1-((IF(ISNUMBER(D24),D24/MAX((F24/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E24),E24/MAX((F24/C7),0.000000001),0))^2)/((IF(ISNUMBER(D24),D24/MAX((F24/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E24),E24/MAX((F24/C7),0.000000001),0))^2))),0),"")</f>
         <v/>
       </c>
-      <c r="I87" s="39" t="str">
+      <c r="I87" s="24" t="str">
         <f aca="false">IF(F24&lt;&gt;"",IFERROR(((IF(ISNUMBER(D24),D24/MAX((F24/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E24),E24/MAX((F24/C7),0.000000001),0))^2)/((IF(ISNUMBER(D24),D24/MAX((F24/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E24),E24/MAX((F24/C7),0.000000001),0))^2)*100,0),"")</f>
         <v/>
       </c>
@@ -2943,122 +3117,122 @@
         <f aca="false">F25</f>
         <v/>
       </c>
-      <c r="E88" s="38" t="str">
+      <c r="E88" s="25" t="str">
         <f aca="false">G25</f>
         <v/>
       </c>
-      <c r="F88" s="39" t="str">
+      <c r="F88" s="24" t="str">
         <f aca="false">IF(F25&lt;&gt;"",IFERROR((1+SQRT(((IF(ISNUMBER(D25),D25/MAX((F25/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E25),E25/MAX((F25/C7),0.000000001),0))^2)/((IF(ISNUMBER(D25),D25/MAX((F25/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E25),E25/MAX((F25/C7),0.000000001),0))^2)))/(1-SQRT(((IF(ISNUMBER(D25),D25/MAX((F25/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E25),E25/MAX((F25/C7),0.000000001),0))^2)/((IF(ISNUMBER(D25),D25/MAX((F25/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E25),E25/MAX((F25/C7),0.000000001),0))^2))),999),"")</f>
         <v/>
       </c>
-      <c r="G88" s="38" t="str">
+      <c r="G88" s="25" t="str">
         <f aca="false">IF(F25&lt;&gt;"",IFERROR(-20*LOG10(MAX(SQRT(((IF(ISNUMBER(D25),D25/MAX((F25/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E25),E25/MAX((F25/C7),0.000000001),0))^2)/((IF(ISNUMBER(D25),D25/MAX((F25/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E25),E25/MAX((F25/C7),0.000000001),0))^2)),0.000000001)),0),"")</f>
         <v/>
       </c>
-      <c r="H88" s="39" t="str">
+      <c r="H88" s="24" t="str">
         <f aca="false">IF(F25&lt;&gt;"",IFERROR(MAX(0,-10*LOG10(1-((IF(ISNUMBER(D25),D25/MAX((F25/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E25),E25/MAX((F25/C7),0.000000001),0))^2)/((IF(ISNUMBER(D25),D25/MAX((F25/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E25),E25/MAX((F25/C7),0.000000001),0))^2))),0),"")</f>
         <v/>
       </c>
-      <c r="I88" s="39" t="str">
+      <c r="I88" s="24" t="str">
         <f aca="false">IF(F25&lt;&gt;"",IFERROR(((IF(ISNUMBER(D25),D25/MAX((F25/C7),0.000000001),C7)-C7)^2+(IF(ISNUMBER(E25),E25/MAX((F25/C7),0.000000001),0))^2)/((IF(ISNUMBER(D25),D25/MAX((F25/C7),0.000000001),C7)+C7)^2+(IF(ISNUMBER(E25),E25/MAX((F25/C7),0.000000001),0))^2)*100,0),"")</f>
         <v/>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B90" s="40" t="s">
+      <c r="B90" s="30" t="s">
         <v>69</v>
       </c>
-      <c r="C90" s="40"/>
-      <c r="D90" s="40"/>
-      <c r="E90" s="40"/>
-      <c r="F90" s="40"/>
-      <c r="G90" s="40"/>
-      <c r="H90" s="40"/>
-      <c r="I90" s="40"/>
+      <c r="C90" s="30"/>
+      <c r="D90" s="30"/>
+      <c r="E90" s="30"/>
+      <c r="F90" s="30"/>
+      <c r="G90" s="30"/>
+      <c r="H90" s="30"/>
+      <c r="I90" s="30"/>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B91" s="41" t="s">
+      <c r="B91" s="31" t="s">
         <v>70</v>
       </c>
-      <c r="C91" s="41"/>
-      <c r="D91" s="41"/>
-      <c r="E91" s="41"/>
-      <c r="F91" s="41"/>
-      <c r="G91" s="41"/>
-      <c r="H91" s="41"/>
-      <c r="I91" s="41"/>
+      <c r="C91" s="31"/>
+      <c r="D91" s="31"/>
+      <c r="E91" s="31"/>
+      <c r="F91" s="31"/>
+      <c r="G91" s="31"/>
+      <c r="H91" s="31"/>
+      <c r="I91" s="31"/>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B92" s="41" t="s">
+      <c r="B92" s="31" t="s">
         <v>71</v>
       </c>
-      <c r="C92" s="41"/>
-      <c r="D92" s="41"/>
-      <c r="E92" s="41"/>
-      <c r="F92" s="41"/>
-      <c r="G92" s="41"/>
-      <c r="H92" s="41"/>
-      <c r="I92" s="41"/>
+      <c r="C92" s="31"/>
+      <c r="D92" s="31"/>
+      <c r="E92" s="31"/>
+      <c r="F92" s="31"/>
+      <c r="G92" s="31"/>
+      <c r="H92" s="31"/>
+      <c r="I92" s="31"/>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B93" s="41" t="s">
+      <c r="B93" s="31" t="s">
         <v>72</v>
       </c>
-      <c r="C93" s="41"/>
-      <c r="D93" s="41"/>
-      <c r="E93" s="41"/>
-      <c r="F93" s="41"/>
-      <c r="G93" s="41"/>
-      <c r="H93" s="41"/>
-      <c r="I93" s="41"/>
+      <c r="C93" s="31"/>
+      <c r="D93" s="31"/>
+      <c r="E93" s="31"/>
+      <c r="F93" s="31"/>
+      <c r="G93" s="31"/>
+      <c r="H93" s="31"/>
+      <c r="I93" s="31"/>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B94" s="41" t="s">
+      <c r="B94" s="31" t="s">
         <v>73</v>
       </c>
-      <c r="C94" s="41"/>
-      <c r="D94" s="41"/>
-      <c r="E94" s="41"/>
-      <c r="F94" s="41"/>
-      <c r="G94" s="41"/>
-      <c r="H94" s="41"/>
-      <c r="I94" s="41"/>
+      <c r="C94" s="31"/>
+      <c r="D94" s="31"/>
+      <c r="E94" s="31"/>
+      <c r="F94" s="31"/>
+      <c r="G94" s="31"/>
+      <c r="H94" s="31"/>
+      <c r="I94" s="31"/>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B95" s="41" t="s">
+      <c r="B95" s="31" t="s">
         <v>74</v>
       </c>
-      <c r="C95" s="41"/>
-      <c r="D95" s="41"/>
-      <c r="E95" s="41"/>
-      <c r="F95" s="41"/>
-      <c r="G95" s="41"/>
-      <c r="H95" s="41"/>
-      <c r="I95" s="41"/>
+      <c r="C95" s="31"/>
+      <c r="D95" s="31"/>
+      <c r="E95" s="31"/>
+      <c r="F95" s="31"/>
+      <c r="G95" s="31"/>
+      <c r="H95" s="31"/>
+      <c r="I95" s="31"/>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B96" s="41" t="s">
+      <c r="B96" s="31" t="s">
         <v>75</v>
       </c>
-      <c r="C96" s="41"/>
-      <c r="D96" s="41"/>
-      <c r="E96" s="41"/>
-      <c r="F96" s="41"/>
-      <c r="G96" s="41"/>
-      <c r="H96" s="41"/>
-      <c r="I96" s="41"/>
+      <c r="C96" s="31"/>
+      <c r="D96" s="31"/>
+      <c r="E96" s="31"/>
+      <c r="F96" s="31"/>
+      <c r="G96" s="31"/>
+      <c r="H96" s="31"/>
+      <c r="I96" s="31"/>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B97" s="41" t="s">
+      <c r="B97" s="31" t="s">
         <v>76</v>
       </c>
-      <c r="C97" s="41"/>
-      <c r="D97" s="41"/>
-      <c r="E97" s="41"/>
-      <c r="F97" s="41"/>
-      <c r="G97" s="41"/>
-      <c r="H97" s="41"/>
-      <c r="I97" s="41"/>
+      <c r="C97" s="31"/>
+      <c r="D97" s="31"/>
+      <c r="E97" s="31"/>
+      <c r="F97" s="31"/>
+      <c r="G97" s="31"/>
+      <c r="H97" s="31"/>
+      <c r="I97" s="31"/>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B99" s="2" t="s">
@@ -3110,7 +3284,7 @@
       <c r="B104" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="C104" s="42" t="n">
+      <c r="C104" s="32" t="n">
         <f aca="false">C9</f>
         <v>16</v>
       </c>
@@ -3127,7 +3301,7 @@
       <c r="B105" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="C105" s="42" t="n">
+      <c r="C105" s="32" t="n">
         <f aca="false">C8</f>
         <v>0.45</v>
       </c>
@@ -3144,7 +3318,7 @@
       <c r="B106" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="C106" s="42" t="n">
+      <c r="C106" s="32" t="n">
         <f aca="false">MAX(C8*1.1,C8+0.05)</f>
         <v>0.5</v>
       </c>
@@ -3204,7 +3378,7 @@
       <c r="B111" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="C111" s="43" t="n">
+      <c r="C111" s="33" t="n">
         <f aca="false">IFERROR(IF(C107&gt;0,(C107-1)*C106+C105,""),"")</f>
         <v>39.95</v>
       </c>
@@ -3221,7 +3395,7 @@
       <c r="B112" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="C112" s="43" t="n">
+      <c r="C112" s="33" t="n">
         <f aca="false">(C104+C105)/2</f>
         <v>8.225</v>
       </c>
@@ -3238,7 +3412,7 @@
       <c r="B113" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="C113" s="43" t="n">
+      <c r="C113" s="33" t="n">
         <f aca="false">((C104+C105)/2)/25.4</f>
         <v>0.323818897637795</v>
       </c>
@@ -3255,7 +3429,7 @@
       <c r="B114" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="C114" s="43" t="n">
+      <c r="C114" s="33" t="n">
         <f aca="false">IFERROR(C111/25.4,"")</f>
         <v>1.57283464566929</v>
       </c>
@@ -3272,7 +3446,7 @@
       <c r="B115" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="C115" s="43" t="n">
+      <c r="C115" s="33" t="n">
         <f aca="false">IFERROR((C113^2*C107^2)/(9*C113+10*C114),"")</f>
         <v>35.9977335339286</v>
       </c>
@@ -3289,7 +3463,7 @@
       <c r="B116" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="C116" s="43" t="n">
+      <c r="C116" s="33" t="n">
         <f aca="false">IFERROR(2*PI()*C32*1000000*C115/1000000,"")</f>
         <v>1628.49909911145</v>
       </c>
@@ -3306,7 +3480,7 @@
       <c r="B117" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="C117" s="43" t="n">
+      <c r="C117" s="33" t="n">
         <f aca="false">IFERROR(4*MIN(F15:F25)/(2*PI()*C32*1000000)*1000000,"")</f>
         <v>17.6838825657662</v>
       </c>
@@ -3323,7 +3497,7 @@
       <c r="B118" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="C118" s="43" t="str">
+      <c r="C118" s="33" t="str">
         <f aca="false">IFERROR(IF(AND(ISNUMBER(C115),ISNUMBER(C117)),IF(C115&gt;=C117,"✔ YES","✘ INCREASE TURNS"),"—"),"")</f>
         <v>✔ YES</v>
       </c>
@@ -3335,6 +3509,649 @@
       </c>
       <c r="F118" s="9"/>
       <c r="G118" s="9"/>
+    </row>
+    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B121" s="34" t="s">
+        <v>108</v>
+      </c>
+      <c r="C121" s="34"/>
+      <c r="D121" s="34"/>
+      <c r="E121" s="34"/>
+      <c r="F121" s="34"/>
+      <c r="G121" s="34"/>
+      <c r="H121" s="34"/>
+      <c r="I121" s="34"/>
+      <c r="J121" s="34"/>
+    </row>
+    <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B122" s="35" t="s">
+        <v>109</v>
+      </c>
+      <c r="C122" s="35"/>
+      <c r="D122" s="35"/>
+      <c r="E122" s="35"/>
+      <c r="F122" s="35"/>
+      <c r="G122" s="35"/>
+      <c r="H122" s="35"/>
+      <c r="I122" s="35"/>
+      <c r="J122" s="35"/>
+    </row>
+    <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B124" s="36" t="s">
+        <v>110</v>
+      </c>
+      <c r="C124" s="36"/>
+      <c r="D124" s="36"/>
+      <c r="E124" s="36"/>
+      <c r="F124" s="36"/>
+      <c r="G124" s="36"/>
+      <c r="H124" s="36"/>
+      <c r="I124" s="36"/>
+      <c r="J124" s="36"/>
+    </row>
+    <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B125" s="37" t="s">
+        <v>111</v>
+      </c>
+      <c r="C125" s="37"/>
+      <c r="D125" s="37"/>
+      <c r="E125" s="37"/>
+      <c r="F125" s="37"/>
+      <c r="G125" s="37"/>
+      <c r="H125" s="37"/>
+      <c r="I125" s="37"/>
+      <c r="J125" s="37"/>
+    </row>
+    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B126" s="37" t="s">
+        <v>112</v>
+      </c>
+      <c r="C126" s="37"/>
+      <c r="D126" s="37"/>
+      <c r="E126" s="37"/>
+      <c r="F126" s="37"/>
+      <c r="G126" s="37"/>
+      <c r="H126" s="37"/>
+      <c r="I126" s="37"/>
+      <c r="J126" s="37"/>
+    </row>
+    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B127" s="37" t="s">
+        <v>113</v>
+      </c>
+      <c r="C127" s="37"/>
+      <c r="D127" s="37"/>
+      <c r="E127" s="37"/>
+      <c r="F127" s="37"/>
+      <c r="G127" s="37"/>
+      <c r="H127" s="37"/>
+      <c r="I127" s="37"/>
+      <c r="J127" s="37"/>
+    </row>
+    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B128" s="37" t="s">
+        <v>114</v>
+      </c>
+      <c r="C128" s="37"/>
+      <c r="D128" s="37"/>
+      <c r="E128" s="37"/>
+      <c r="F128" s="37"/>
+      <c r="G128" s="37"/>
+      <c r="H128" s="37"/>
+      <c r="I128" s="37"/>
+      <c r="J128" s="37"/>
+    </row>
+    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B129" s="37" t="s">
+        <v>115</v>
+      </c>
+      <c r="C129" s="37"/>
+      <c r="D129" s="37"/>
+      <c r="E129" s="37"/>
+      <c r="F129" s="37"/>
+      <c r="G129" s="37"/>
+      <c r="H129" s="37"/>
+      <c r="I129" s="37"/>
+      <c r="J129" s="37"/>
+    </row>
+    <row r="131" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B131" s="38" t="s">
+        <v>21</v>
+      </c>
+      <c r="C131" s="38" t="s">
+        <v>116</v>
+      </c>
+      <c r="D131" s="38" t="s">
+        <v>117</v>
+      </c>
+      <c r="E131" s="38" t="s">
+        <v>118</v>
+      </c>
+      <c r="F131" s="38" t="s">
+        <v>119</v>
+      </c>
+      <c r="G131" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="H131" s="38" t="s">
+        <v>121</v>
+      </c>
+      <c r="I131" s="38" t="s">
+        <v>122</v>
+      </c>
+      <c r="J131" s="38" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B132" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="C132" s="40" t="n">
+        <f aca="false">C15</f>
+        <v>7.2</v>
+      </c>
+      <c r="D132" s="40" t="n">
+        <f aca="false">D15</f>
+        <v>200</v>
+      </c>
+      <c r="E132" s="40" t="n">
+        <f aca="false">IF(ISNUMBER(E15),E15,"—")</f>
+        <v>0</v>
+      </c>
+      <c r="F132" s="40" t="n">
+        <f aca="false">IF(ISNUMBER(G15),G15,"—")</f>
+        <v>0</v>
+      </c>
+      <c r="G132" s="41" t="str">
+        <f aca="false">IFERROR(IF(AND(H15="YES",ISNUMBER(F15),F15&gt;0,ISNUMBER(D15),D15&gt;0),IF(($C$7*IF(ISNUMBER(E15),E15,0)/F15)&gt;0,($C$7*IF(ISNUMBER(E15),E15,0)/F15)/(2*PI()*C15*1000000)*1000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+      <c r="H132" s="40" t="str">
+        <f aca="false">IFERROR(IF(AND(H15="YES",ISNUMBER(F15),F15&gt;0,ISNUMBER(D15),D15&gt;0),IF(($C$7*IF(ISNUMBER(E15),E15,0)/F15)&lt;0,1/((2*PI()*C15*1000000)*ABS(($C$7*IF(ISNUMBER(E15),E15,0)/F15)))*1000000000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+      <c r="I132" s="41" t="str">
+        <f aca="false">IFERROR(IF(AND(H15="YES",ISNUMBER(F15),F15&gt;0,ISNUMBER(D15),D15&gt;0),IF((F15*IF(ISNUMBER(E15),E15,0)/($C$7*(D15^2+IF(ISNUMBER(E15),E15,0)^2)))&lt;0,-1/((2*PI()*C15*1000000)*(F15*IF(ISNUMBER(E15),E15,0)/($C$7*(D15^2+IF(ISNUMBER(E15),E15,0)^2))))*1000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+      <c r="J132" s="40" t="str">
+        <f aca="false">IFERROR(IF(AND(H15="YES",ISNUMBER(F15),F15&gt;0,ISNUMBER(D15),D15&gt;0),IF((F15*IF(ISNUMBER(E15),E15,0)/($C$7*(D15^2+IF(ISNUMBER(E15),E15,0)^2)))&gt;0,(F15*IF(ISNUMBER(E15),E15,0)/($C$7*(D15^2+IF(ISNUMBER(E15),E15,0)^2)))/(2*PI()*C15*1000000)*1000000000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B133" s="42" t="n">
+        <v>2</v>
+      </c>
+      <c r="C133" s="43" t="n">
+        <f aca="false">C16</f>
+        <v>10</v>
+      </c>
+      <c r="D133" s="43" t="n">
+        <f aca="false">D16</f>
+        <v>300</v>
+      </c>
+      <c r="E133" s="43" t="n">
+        <f aca="false">IF(ISNUMBER(E16),E16,"—")</f>
+        <v>100</v>
+      </c>
+      <c r="F133" s="43" t="n">
+        <f aca="false">IF(ISNUMBER(G16),G16,"—")</f>
+        <v>18.434948822922</v>
+      </c>
+      <c r="G133" s="44" t="n">
+        <f aca="false">IFERROR(IF(AND(H16="YES",ISNUMBER(F16),F16&gt;0,ISNUMBER(D16),D16&gt;0),IF(($C$7*IF(ISNUMBER(E16),E16,0)/F16)&gt;0,($C$7*IF(ISNUMBER(E16),E16,0)/F16)/(2*PI()*C16*1000000)*1000000,"—"),"—"),"—")</f>
+        <v>0.251646060522435</v>
+      </c>
+      <c r="H133" s="43" t="str">
+        <f aca="false">IFERROR(IF(AND(H16="YES",ISNUMBER(F16),F16&gt;0,ISNUMBER(D16),D16&gt;0),IF(($C$7*IF(ISNUMBER(E16),E16,0)/F16)&lt;0,1/((2*PI()*C16*1000000)*ABS(($C$7*IF(ISNUMBER(E16),E16,0)/F16)))*1000000000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+      <c r="I133" s="44" t="str">
+        <f aca="false">IFERROR(IF(AND(H16="YES",ISNUMBER(F16),F16&gt;0,ISNUMBER(D16),D16&gt;0),IF((F16*IF(ISNUMBER(E16),E16,0)/($C$7*(D16^2+IF(ISNUMBER(E16),E16,0)^2)))&lt;0,-1/((2*PI()*C16*1000000)*(F16*IF(ISNUMBER(E16),E16,0)/($C$7*(D16^2+IF(ISNUMBER(E16),E16,0)^2))))*1000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+      <c r="J133" s="43" t="n">
+        <f aca="false">IFERROR(IF(AND(H16="YES",ISNUMBER(F16),F16&gt;0,ISNUMBER(D16),D16&gt;0),IF((F16*IF(ISNUMBER(E16),E16,0)/($C$7*(D16^2+IF(ISNUMBER(E16),E16,0)^2)))&gt;0,(F16*IF(ISNUMBER(E16),E16,0)/($C$7*(D16^2+IF(ISNUMBER(E16),E16,0)^2)))/(2*PI()*C16*1000000)*1000000000000,"—"),"—"),"—")</f>
+        <v>100.658424208974</v>
+      </c>
+    </row>
+    <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B134" s="39" t="n">
+        <v>3</v>
+      </c>
+      <c r="C134" s="40" t="n">
+        <f aca="false">C17</f>
+        <v>18</v>
+      </c>
+      <c r="D134" s="40" t="n">
+        <f aca="false">D17</f>
+        <v>450</v>
+      </c>
+      <c r="E134" s="40" t="n">
+        <f aca="false">IF(ISNUMBER(E17),E17,"—")</f>
+        <v>-80</v>
+      </c>
+      <c r="F134" s="40" t="n">
+        <f aca="false">IF(ISNUMBER(G17),G17,"—")</f>
+        <v>-10.0805979875423</v>
+      </c>
+      <c r="G134" s="41" t="str">
+        <f aca="false">IFERROR(IF(AND(H17="YES",ISNUMBER(F17),F17&gt;0,ISNUMBER(D17),D17&gt;0),IF(($C$7*IF(ISNUMBER(E17),E17,0)/F17)&gt;0,($C$7*IF(ISNUMBER(E17),E17,0)/F17)/(2*PI()*C17*1000000)*1000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+      <c r="H134" s="40" t="n">
+        <f aca="false">IFERROR(IF(AND(H17="YES",ISNUMBER(F17),F17&gt;0,ISNUMBER(D17),D17&gt;0),IF(($C$7*IF(ISNUMBER(E17),E17,0)/F17)&lt;0,1/((2*PI()*C17*1000000)*ABS(($C$7*IF(ISNUMBER(E17),E17,0)/F17)))*1000000000000,"—"),"—"),"—")</f>
+        <v>1010.31512621913</v>
+      </c>
+      <c r="I134" s="41" t="n">
+        <f aca="false">IFERROR(IF(AND(H17="YES",ISNUMBER(F17),F17&gt;0,ISNUMBER(D17),D17&gt;0),IF((F17*IF(ISNUMBER(E17),E17,0)/($C$7*(D17^2+IF(ISNUMBER(E17),E17,0)^2)))&lt;0,-1/((2*PI()*C17*1000000)*(F17*IF(ISNUMBER(E17),E17,0)/($C$7*(D17^2+IF(ISNUMBER(E17),E17,0)^2))))*1000000,"—"),"—"),"—")</f>
+        <v>2.52578781554784</v>
+      </c>
+      <c r="J134" s="40" t="str">
+        <f aca="false">IFERROR(IF(AND(H17="YES",ISNUMBER(F17),F17&gt;0,ISNUMBER(D17),D17&gt;0),IF((F17*IF(ISNUMBER(E17),E17,0)/($C$7*(D17^2+IF(ISNUMBER(E17),E17,0)^2)))&gt;0,(F17*IF(ISNUMBER(E17),E17,0)/($C$7*(D17^2+IF(ISNUMBER(E17),E17,0)^2)))/(2*PI()*C17*1000000)*1000000000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B135" s="42" t="n">
+        <v>4</v>
+      </c>
+      <c r="C135" s="43" t="n">
+        <f aca="false">C18</f>
+        <v>28</v>
+      </c>
+      <c r="D135" s="43" t="n">
+        <f aca="false">D18</f>
+        <v>800</v>
+      </c>
+      <c r="E135" s="43" t="n">
+        <f aca="false">IF(ISNUMBER(E18),E18,"—")</f>
+        <v>0</v>
+      </c>
+      <c r="F135" s="43" t="n">
+        <f aca="false">IF(ISNUMBER(G18),G18,"—")</f>
+        <v>0</v>
+      </c>
+      <c r="G135" s="44" t="str">
+        <f aca="false">IFERROR(IF(AND(H18="YES",ISNUMBER(F18),F18&gt;0,ISNUMBER(D18),D18&gt;0),IF(($C$7*IF(ISNUMBER(E18),E18,0)/F18)&gt;0,($C$7*IF(ISNUMBER(E18),E18,0)/F18)/(2*PI()*C18*1000000)*1000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+      <c r="H135" s="43" t="str">
+        <f aca="false">IFERROR(IF(AND(H18="YES",ISNUMBER(F18),F18&gt;0,ISNUMBER(D18),D18&gt;0),IF(($C$7*IF(ISNUMBER(E18),E18,0)/F18)&lt;0,1/((2*PI()*C18*1000000)*ABS(($C$7*IF(ISNUMBER(E18),E18,0)/F18)))*1000000000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+      <c r="I135" s="44" t="str">
+        <f aca="false">IFERROR(IF(AND(H18="YES",ISNUMBER(F18),F18&gt;0,ISNUMBER(D18),D18&gt;0),IF((F18*IF(ISNUMBER(E18),E18,0)/($C$7*(D18^2+IF(ISNUMBER(E18),E18,0)^2)))&lt;0,-1/((2*PI()*C18*1000000)*(F18*IF(ISNUMBER(E18),E18,0)/($C$7*(D18^2+IF(ISNUMBER(E18),E18,0)^2))))*1000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+      <c r="J135" s="43" t="str">
+        <f aca="false">IFERROR(IF(AND(H18="YES",ISNUMBER(F18),F18&gt;0,ISNUMBER(D18),D18&gt;0),IF((F18*IF(ISNUMBER(E18),E18,0)/($C$7*(D18^2+IF(ISNUMBER(E18),E18,0)^2)))&gt;0,(F18*IF(ISNUMBER(E18),E18,0)/($C$7*(D18^2+IF(ISNUMBER(E18),E18,0)^2)))/(2*PI()*C18*1000000)*1000000000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B136" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="C136" s="40" t="n">
+        <f aca="false">C19</f>
+        <v>0</v>
+      </c>
+      <c r="D136" s="40" t="n">
+        <f aca="false">D19</f>
+        <v>0</v>
+      </c>
+      <c r="E136" s="40" t="str">
+        <f aca="false">IF(ISNUMBER(E19),E19,"—")</f>
+        <v>—</v>
+      </c>
+      <c r="F136" s="40" t="str">
+        <f aca="false">IF(ISNUMBER(G19),G19,"—")</f>
+        <v>—</v>
+      </c>
+      <c r="G136" s="41" t="str">
+        <f aca="false">IFERROR(IF(AND(H19="YES",ISNUMBER(F19),F19&gt;0,ISNUMBER(D19),D19&gt;0),IF(($C$7*IF(ISNUMBER(E19),E19,0)/F19)&gt;0,($C$7*IF(ISNUMBER(E19),E19,0)/F19)/(2*PI()*C19*1000000)*1000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+      <c r="H136" s="40" t="str">
+        <f aca="false">IFERROR(IF(AND(H19="YES",ISNUMBER(F19),F19&gt;0,ISNUMBER(D19),D19&gt;0),IF(($C$7*IF(ISNUMBER(E19),E19,0)/F19)&lt;0,1/((2*PI()*C19*1000000)*ABS(($C$7*IF(ISNUMBER(E19),E19,0)/F19)))*1000000000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+      <c r="I136" s="41" t="str">
+        <f aca="false">IFERROR(IF(AND(H19="YES",ISNUMBER(F19),F19&gt;0,ISNUMBER(D19),D19&gt;0),IF((F19*IF(ISNUMBER(E19),E19,0)/($C$7*(D19^2+IF(ISNUMBER(E19),E19,0)^2)))&lt;0,-1/((2*PI()*C19*1000000)*(F19*IF(ISNUMBER(E19),E19,0)/($C$7*(D19^2+IF(ISNUMBER(E19),E19,0)^2))))*1000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+      <c r="J136" s="40" t="str">
+        <f aca="false">IFERROR(IF(AND(H19="YES",ISNUMBER(F19),F19&gt;0,ISNUMBER(D19),D19&gt;0),IF((F19*IF(ISNUMBER(E19),E19,0)/($C$7*(D19^2+IF(ISNUMBER(E19),E19,0)^2)))&gt;0,(F19*IF(ISNUMBER(E19),E19,0)/($C$7*(D19^2+IF(ISNUMBER(E19),E19,0)^2)))/(2*PI()*C19*1000000)*1000000000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B137" s="42" t="n">
+        <v>6</v>
+      </c>
+      <c r="C137" s="43" t="n">
+        <f aca="false">C20</f>
+        <v>0</v>
+      </c>
+      <c r="D137" s="43" t="n">
+        <f aca="false">D20</f>
+        <v>0</v>
+      </c>
+      <c r="E137" s="43" t="str">
+        <f aca="false">IF(ISNUMBER(E20),E20,"—")</f>
+        <v>—</v>
+      </c>
+      <c r="F137" s="43" t="str">
+        <f aca="false">IF(ISNUMBER(G20),G20,"—")</f>
+        <v>—</v>
+      </c>
+      <c r="G137" s="44" t="str">
+        <f aca="false">IFERROR(IF(AND(H20="YES",ISNUMBER(F20),F20&gt;0,ISNUMBER(D20),D20&gt;0),IF(($C$7*IF(ISNUMBER(E20),E20,0)/F20)&gt;0,($C$7*IF(ISNUMBER(E20),E20,0)/F20)/(2*PI()*C20*1000000)*1000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+      <c r="H137" s="43" t="str">
+        <f aca="false">IFERROR(IF(AND(H20="YES",ISNUMBER(F20),F20&gt;0,ISNUMBER(D20),D20&gt;0),IF(($C$7*IF(ISNUMBER(E20),E20,0)/F20)&lt;0,1/((2*PI()*C20*1000000)*ABS(($C$7*IF(ISNUMBER(E20),E20,0)/F20)))*1000000000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+      <c r="I137" s="44" t="str">
+        <f aca="false">IFERROR(IF(AND(H20="YES",ISNUMBER(F20),F20&gt;0,ISNUMBER(D20),D20&gt;0),IF((F20*IF(ISNUMBER(E20),E20,0)/($C$7*(D20^2+IF(ISNUMBER(E20),E20,0)^2)))&lt;0,-1/((2*PI()*C20*1000000)*(F20*IF(ISNUMBER(E20),E20,0)/($C$7*(D20^2+IF(ISNUMBER(E20),E20,0)^2))))*1000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+      <c r="J137" s="43" t="str">
+        <f aca="false">IFERROR(IF(AND(H20="YES",ISNUMBER(F20),F20&gt;0,ISNUMBER(D20),D20&gt;0),IF((F20*IF(ISNUMBER(E20),E20,0)/($C$7*(D20^2+IF(ISNUMBER(E20),E20,0)^2)))&gt;0,(F20*IF(ISNUMBER(E20),E20,0)/($C$7*(D20^2+IF(ISNUMBER(E20),E20,0)^2)))/(2*PI()*C20*1000000)*1000000000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B138" s="39" t="n">
+        <v>7</v>
+      </c>
+      <c r="C138" s="40" t="n">
+        <f aca="false">C21</f>
+        <v>0</v>
+      </c>
+      <c r="D138" s="40" t="n">
+        <f aca="false">D21</f>
+        <v>0</v>
+      </c>
+      <c r="E138" s="40" t="str">
+        <f aca="false">IF(ISNUMBER(E21),E21,"—")</f>
+        <v>—</v>
+      </c>
+      <c r="F138" s="40" t="str">
+        <f aca="false">IF(ISNUMBER(G21),G21,"—")</f>
+        <v>—</v>
+      </c>
+      <c r="G138" s="41" t="str">
+        <f aca="false">IFERROR(IF(AND(H21="YES",ISNUMBER(F21),F21&gt;0,ISNUMBER(D21),D21&gt;0),IF(($C$7*IF(ISNUMBER(E21),E21,0)/F21)&gt;0,($C$7*IF(ISNUMBER(E21),E21,0)/F21)/(2*PI()*C21*1000000)*1000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+      <c r="H138" s="40" t="str">
+        <f aca="false">IFERROR(IF(AND(H21="YES",ISNUMBER(F21),F21&gt;0,ISNUMBER(D21),D21&gt;0),IF(($C$7*IF(ISNUMBER(E21),E21,0)/F21)&lt;0,1/((2*PI()*C21*1000000)*ABS(($C$7*IF(ISNUMBER(E21),E21,0)/F21)))*1000000000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+      <c r="I138" s="41" t="str">
+        <f aca="false">IFERROR(IF(AND(H21="YES",ISNUMBER(F21),F21&gt;0,ISNUMBER(D21),D21&gt;0),IF((F21*IF(ISNUMBER(E21),E21,0)/($C$7*(D21^2+IF(ISNUMBER(E21),E21,0)^2)))&lt;0,-1/((2*PI()*C21*1000000)*(F21*IF(ISNUMBER(E21),E21,0)/($C$7*(D21^2+IF(ISNUMBER(E21),E21,0)^2))))*1000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+      <c r="J138" s="40" t="str">
+        <f aca="false">IFERROR(IF(AND(H21="YES",ISNUMBER(F21),F21&gt;0,ISNUMBER(D21),D21&gt;0),IF((F21*IF(ISNUMBER(E21),E21,0)/($C$7*(D21^2+IF(ISNUMBER(E21),E21,0)^2)))&gt;0,(F21*IF(ISNUMBER(E21),E21,0)/($C$7*(D21^2+IF(ISNUMBER(E21),E21,0)^2)))/(2*PI()*C21*1000000)*1000000000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B139" s="42" t="n">
+        <v>8</v>
+      </c>
+      <c r="C139" s="43" t="n">
+        <f aca="false">C22</f>
+        <v>0</v>
+      </c>
+      <c r="D139" s="43" t="n">
+        <f aca="false">D22</f>
+        <v>0</v>
+      </c>
+      <c r="E139" s="43" t="str">
+        <f aca="false">IF(ISNUMBER(E22),E22,"—")</f>
+        <v>—</v>
+      </c>
+      <c r="F139" s="43" t="str">
+        <f aca="false">IF(ISNUMBER(G22),G22,"—")</f>
+        <v>—</v>
+      </c>
+      <c r="G139" s="44" t="str">
+        <f aca="false">IFERROR(IF(AND(H22="YES",ISNUMBER(F22),F22&gt;0,ISNUMBER(D22),D22&gt;0),IF(($C$7*IF(ISNUMBER(E22),E22,0)/F22)&gt;0,($C$7*IF(ISNUMBER(E22),E22,0)/F22)/(2*PI()*C22*1000000)*1000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+      <c r="H139" s="43" t="str">
+        <f aca="false">IFERROR(IF(AND(H22="YES",ISNUMBER(F22),F22&gt;0,ISNUMBER(D22),D22&gt;0),IF(($C$7*IF(ISNUMBER(E22),E22,0)/F22)&lt;0,1/((2*PI()*C22*1000000)*ABS(($C$7*IF(ISNUMBER(E22),E22,0)/F22)))*1000000000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+      <c r="I139" s="44" t="str">
+        <f aca="false">IFERROR(IF(AND(H22="YES",ISNUMBER(F22),F22&gt;0,ISNUMBER(D22),D22&gt;0),IF((F22*IF(ISNUMBER(E22),E22,0)/($C$7*(D22^2+IF(ISNUMBER(E22),E22,0)^2)))&lt;0,-1/((2*PI()*C22*1000000)*(F22*IF(ISNUMBER(E22),E22,0)/($C$7*(D22^2+IF(ISNUMBER(E22),E22,0)^2))))*1000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+      <c r="J139" s="43" t="str">
+        <f aca="false">IFERROR(IF(AND(H22="YES",ISNUMBER(F22),F22&gt;0,ISNUMBER(D22),D22&gt;0),IF((F22*IF(ISNUMBER(E22),E22,0)/($C$7*(D22^2+IF(ISNUMBER(E22),E22,0)^2)))&gt;0,(F22*IF(ISNUMBER(E22),E22,0)/($C$7*(D22^2+IF(ISNUMBER(E22),E22,0)^2)))/(2*PI()*C22*1000000)*1000000000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B140" s="39" t="n">
+        <v>9</v>
+      </c>
+      <c r="C140" s="40" t="n">
+        <f aca="false">C23</f>
+        <v>0</v>
+      </c>
+      <c r="D140" s="40" t="n">
+        <f aca="false">D23</f>
+        <v>0</v>
+      </c>
+      <c r="E140" s="40" t="str">
+        <f aca="false">IF(ISNUMBER(E23),E23,"—")</f>
+        <v>—</v>
+      </c>
+      <c r="F140" s="40" t="str">
+        <f aca="false">IF(ISNUMBER(G23),G23,"—")</f>
+        <v>—</v>
+      </c>
+      <c r="G140" s="41" t="str">
+        <f aca="false">IFERROR(IF(AND(H23="YES",ISNUMBER(F23),F23&gt;0,ISNUMBER(D23),D23&gt;0),IF(($C$7*IF(ISNUMBER(E23),E23,0)/F23)&gt;0,($C$7*IF(ISNUMBER(E23),E23,0)/F23)/(2*PI()*C23*1000000)*1000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+      <c r="H140" s="40" t="str">
+        <f aca="false">IFERROR(IF(AND(H23="YES",ISNUMBER(F23),F23&gt;0,ISNUMBER(D23),D23&gt;0),IF(($C$7*IF(ISNUMBER(E23),E23,0)/F23)&lt;0,1/((2*PI()*C23*1000000)*ABS(($C$7*IF(ISNUMBER(E23),E23,0)/F23)))*1000000000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+      <c r="I140" s="41" t="str">
+        <f aca="false">IFERROR(IF(AND(H23="YES",ISNUMBER(F23),F23&gt;0,ISNUMBER(D23),D23&gt;0),IF((F23*IF(ISNUMBER(E23),E23,0)/($C$7*(D23^2+IF(ISNUMBER(E23),E23,0)^2)))&lt;0,-1/((2*PI()*C23*1000000)*(F23*IF(ISNUMBER(E23),E23,0)/($C$7*(D23^2+IF(ISNUMBER(E23),E23,0)^2))))*1000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+      <c r="J140" s="40" t="str">
+        <f aca="false">IFERROR(IF(AND(H23="YES",ISNUMBER(F23),F23&gt;0,ISNUMBER(D23),D23&gt;0),IF((F23*IF(ISNUMBER(E23),E23,0)/($C$7*(D23^2+IF(ISNUMBER(E23),E23,0)^2)))&gt;0,(F23*IF(ISNUMBER(E23),E23,0)/($C$7*(D23^2+IF(ISNUMBER(E23),E23,0)^2)))/(2*PI()*C23*1000000)*1000000000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B141" s="42" t="n">
+        <v>10</v>
+      </c>
+      <c r="C141" s="43" t="n">
+        <f aca="false">C24</f>
+        <v>0</v>
+      </c>
+      <c r="D141" s="43" t="n">
+        <f aca="false">D24</f>
+        <v>0</v>
+      </c>
+      <c r="E141" s="43" t="str">
+        <f aca="false">IF(ISNUMBER(E24),E24,"—")</f>
+        <v>—</v>
+      </c>
+      <c r="F141" s="43" t="str">
+        <f aca="false">IF(ISNUMBER(G24),G24,"—")</f>
+        <v>—</v>
+      </c>
+      <c r="G141" s="44" t="str">
+        <f aca="false">IFERROR(IF(AND(H24="YES",ISNUMBER(F24),F24&gt;0,ISNUMBER(D24),D24&gt;0),IF(($C$7*IF(ISNUMBER(E24),E24,0)/F24)&gt;0,($C$7*IF(ISNUMBER(E24),E24,0)/F24)/(2*PI()*C24*1000000)*1000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+      <c r="H141" s="43" t="str">
+        <f aca="false">IFERROR(IF(AND(H24="YES",ISNUMBER(F24),F24&gt;0,ISNUMBER(D24),D24&gt;0),IF(($C$7*IF(ISNUMBER(E24),E24,0)/F24)&lt;0,1/((2*PI()*C24*1000000)*ABS(($C$7*IF(ISNUMBER(E24),E24,0)/F24)))*1000000000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+      <c r="I141" s="44" t="str">
+        <f aca="false">IFERROR(IF(AND(H24="YES",ISNUMBER(F24),F24&gt;0,ISNUMBER(D24),D24&gt;0),IF((F24*IF(ISNUMBER(E24),E24,0)/($C$7*(D24^2+IF(ISNUMBER(E24),E24,0)^2)))&lt;0,-1/((2*PI()*C24*1000000)*(F24*IF(ISNUMBER(E24),E24,0)/($C$7*(D24^2+IF(ISNUMBER(E24),E24,0)^2))))*1000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+      <c r="J141" s="43" t="str">
+        <f aca="false">IFERROR(IF(AND(H24="YES",ISNUMBER(F24),F24&gt;0,ISNUMBER(D24),D24&gt;0),IF((F24*IF(ISNUMBER(E24),E24,0)/($C$7*(D24^2+IF(ISNUMBER(E24),E24,0)^2)))&gt;0,(F24*IF(ISNUMBER(E24),E24,0)/($C$7*(D24^2+IF(ISNUMBER(E24),E24,0)^2)))/(2*PI()*C24*1000000)*1000000000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B142" s="39" t="n">
+        <v>11</v>
+      </c>
+      <c r="C142" s="40" t="n">
+        <f aca="false">C25</f>
+        <v>0</v>
+      </c>
+      <c r="D142" s="40" t="n">
+        <f aca="false">D25</f>
+        <v>0</v>
+      </c>
+      <c r="E142" s="40" t="str">
+        <f aca="false">IF(ISNUMBER(E25),E25,"—")</f>
+        <v>—</v>
+      </c>
+      <c r="F142" s="40" t="str">
+        <f aca="false">IF(ISNUMBER(G25),G25,"—")</f>
+        <v>—</v>
+      </c>
+      <c r="G142" s="41" t="str">
+        <f aca="false">IFERROR(IF(AND(H25="YES",ISNUMBER(F25),F25&gt;0,ISNUMBER(D25),D25&gt;0),IF(($C$7*IF(ISNUMBER(E25),E25,0)/F25)&gt;0,($C$7*IF(ISNUMBER(E25),E25,0)/F25)/(2*PI()*C25*1000000)*1000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+      <c r="H142" s="40" t="str">
+        <f aca="false">IFERROR(IF(AND(H25="YES",ISNUMBER(F25),F25&gt;0,ISNUMBER(D25),D25&gt;0),IF(($C$7*IF(ISNUMBER(E25),E25,0)/F25)&lt;0,1/((2*PI()*C25*1000000)*ABS(($C$7*IF(ISNUMBER(E25),E25,0)/F25)))*1000000000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+      <c r="I142" s="41" t="str">
+        <f aca="false">IFERROR(IF(AND(H25="YES",ISNUMBER(F25),F25&gt;0,ISNUMBER(D25),D25&gt;0),IF((F25*IF(ISNUMBER(E25),E25,0)/($C$7*(D25^2+IF(ISNUMBER(E25),E25,0)^2)))&lt;0,-1/((2*PI()*C25*1000000)*(F25*IF(ISNUMBER(E25),E25,0)/($C$7*(D25^2+IF(ISNUMBER(E25),E25,0)^2))))*1000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+      <c r="J142" s="40" t="str">
+        <f aca="false">IFERROR(IF(AND(H25="YES",ISNUMBER(F25),F25&gt;0,ISNUMBER(D25),D25&gt;0),IF((F25*IF(ISNUMBER(E25),E25,0)/($C$7*(D25^2+IF(ISNUMBER(E25),E25,0)^2)))&gt;0,(F25*IF(ISNUMBER(E25),E25,0)/($C$7*(D25^2+IF(ISNUMBER(E25),E25,0)^2)))/(2*PI()*C25*1000000)*1000000000000,"—"),"—"),"—")</f>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B144" s="36" t="s">
+        <v>124</v>
+      </c>
+      <c r="C144" s="36"/>
+      <c r="D144" s="36"/>
+      <c r="E144" s="36"/>
+      <c r="F144" s="36"/>
+      <c r="G144" s="36"/>
+      <c r="H144" s="36"/>
+      <c r="I144" s="36"/>
+      <c r="J144" s="36"/>
+    </row>
+    <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B145" s="45" t="s">
+        <v>125</v>
+      </c>
+      <c r="C145" s="37" t="s">
+        <v>126</v>
+      </c>
+      <c r="D145" s="37"/>
+      <c r="E145" s="37"/>
+      <c r="F145" s="37"/>
+      <c r="G145" s="37"/>
+      <c r="H145" s="37"/>
+      <c r="I145" s="37"/>
+      <c r="J145" s="37"/>
+    </row>
+    <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B146" s="45" t="s">
+        <v>127</v>
+      </c>
+      <c r="C146" s="37" t="s">
+        <v>128</v>
+      </c>
+      <c r="D146" s="37"/>
+      <c r="E146" s="37"/>
+      <c r="F146" s="37"/>
+      <c r="G146" s="37"/>
+      <c r="H146" s="37"/>
+      <c r="I146" s="37"/>
+      <c r="J146" s="37"/>
+    </row>
+    <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B147" s="45" t="s">
+        <v>129</v>
+      </c>
+      <c r="C147" s="37" t="s">
+        <v>130</v>
+      </c>
+      <c r="D147" s="37"/>
+      <c r="E147" s="37"/>
+      <c r="F147" s="37"/>
+      <c r="G147" s="37"/>
+      <c r="H147" s="37"/>
+      <c r="I147" s="37"/>
+      <c r="J147" s="37"/>
+    </row>
+    <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B148" s="45" t="s">
+        <v>131</v>
+      </c>
+      <c r="C148" s="37" t="s">
+        <v>132</v>
+      </c>
+      <c r="D148" s="37"/>
+      <c r="E148" s="37"/>
+      <c r="F148" s="37"/>
+      <c r="G148" s="37"/>
+      <c r="H148" s="37"/>
+      <c r="I148" s="37"/>
+      <c r="J148" s="37"/>
+    </row>
+    <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B149" s="45" t="s">
+        <v>133</v>
+      </c>
+      <c r="C149" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="D149" s="37"/>
+      <c r="E149" s="37"/>
+      <c r="F149" s="37"/>
+      <c r="G149" s="37"/>
+      <c r="H149" s="37"/>
+      <c r="I149" s="37"/>
+      <c r="J149" s="37"/>
+    </row>
+    <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B150" s="45" t="s">
+        <v>135</v>
+      </c>
+      <c r="C150" s="37" t="s">
+        <v>136</v>
+      </c>
+      <c r="D150" s="37"/>
+      <c r="E150" s="37"/>
+      <c r="F150" s="37"/>
+      <c r="G150" s="37"/>
+      <c r="H150" s="37"/>
+      <c r="I150" s="37"/>
+      <c r="J150" s="37"/>
     </row>
     <row r="1048554" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1048555" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -3360,7 +4177,7 @@
     <row r="1048575" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="47">
+  <mergeCells count="62">
     <mergeCell ref="B2:I2"/>
     <mergeCell ref="B3:I3"/>
     <mergeCell ref="B5:I5"/>
@@ -3408,6 +4225,21 @@
     <mergeCell ref="E116:G116"/>
     <mergeCell ref="E117:G117"/>
     <mergeCell ref="E118:G118"/>
+    <mergeCell ref="B121:J121"/>
+    <mergeCell ref="B122:J122"/>
+    <mergeCell ref="B124:J124"/>
+    <mergeCell ref="B125:J125"/>
+    <mergeCell ref="B126:J126"/>
+    <mergeCell ref="B127:J127"/>
+    <mergeCell ref="B128:J128"/>
+    <mergeCell ref="B129:J129"/>
+    <mergeCell ref="B144:J144"/>
+    <mergeCell ref="C145:J145"/>
+    <mergeCell ref="C146:J146"/>
+    <mergeCell ref="C147:J147"/>
+    <mergeCell ref="C148:J148"/>
+    <mergeCell ref="C149:J149"/>
+    <mergeCell ref="C150:J150"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>